<commit_message>
feat(Début du Code): Rédaction du début des méthodes de déplacement des ennemis et de placement de tours
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0F2457-4C74-4942-A4A5-CC02AB956A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E1F62A-9799-42D4-9C7B-35B8179E7C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-345" yWindow="3030" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="34">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -149,6 +149,9 @@
   </si>
   <si>
     <t>Création du fichier et début de la rédaction du code</t>
+  </si>
+  <si>
+    <t>Création et début de rédaction des méthodes pour le choix de tours et déplacement d'ennemi</t>
   </si>
 </sst>
 </file>
@@ -493,6 +496,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -510,18 +525,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -856,10 +859,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="33"/>
+      <c r="C1" s="28"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -869,10 +872,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="28"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -884,10 +887,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="28"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -899,12 +902,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -927,7 +930,7 @@
       <c r="A6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="28"/>
+      <c r="B6" s="32"/>
       <c r="C6" s="5">
         <v>3</v>
       </c>
@@ -940,7 +943,7 @@
       <c r="A7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="33"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -953,7 +956,7 @@
       <c r="A8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="8">
         <v>3</v>
       </c>
@@ -966,7 +969,7 @@
       <c r="A9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="33"/>
       <c r="C9" s="8">
         <v>1</v>
       </c>
@@ -979,7 +982,7 @@
       <c r="A10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="29"/>
+      <c r="B10" s="33"/>
       <c r="C10" s="10">
         <v>2</v>
       </c>
@@ -992,7 +995,7 @@
       <c r="A11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="29"/>
+      <c r="B11" s="33"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1004,42 +1007,48 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="30"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="25"/>
       <c r="D12" s="26"/>
       <c r="E12" s="27"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="6"/>
+      <c r="A13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="32"/>
+      <c r="C13" s="5">
+        <v>6</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>33</v>
+      </c>
       <c r="E13" s="21"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
-      <c r="B14" s="29"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="8"/>
       <c r="D14" s="9"/>
       <c r="E14" s="8"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
-      <c r="B15" s="29"/>
+      <c r="B15" s="33"/>
       <c r="C15" s="8"/>
       <c r="D15" s="9"/>
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
-      <c r="B16" s="29"/>
+      <c r="B16" s="33"/>
       <c r="C16" s="8"/>
       <c r="D16" s="9"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
-      <c r="B17" s="29"/>
+      <c r="B17" s="33"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1048,10 +1057,10 @@
       <c r="A18" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="29"/>
+      <c r="B18" s="33"/>
       <c r="C18" s="22">
         <f>SUM(C13:C17)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D18" s="23"/>
       <c r="E18" s="24"/>
@@ -1060,42 +1069,42 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="30"/>
+      <c r="B19" s="34"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
       <c r="E19" s="27"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
-      <c r="B20" s="28"/>
+      <c r="B20" s="32"/>
       <c r="C20" s="5"/>
       <c r="D20" s="6"/>
       <c r="E20" s="21"/>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="29"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="8"/>
       <c r="D21" s="9"/>
       <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="29"/>
+      <c r="B22" s="33"/>
       <c r="C22" s="8"/>
       <c r="D22" s="9"/>
       <c r="E22" s="8"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="29"/>
+      <c r="B23" s="33"/>
       <c r="C23" s="8"/>
       <c r="D23" s="9"/>
       <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
-      <c r="B24" s="29"/>
+      <c r="B24" s="33"/>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
       <c r="E24" s="10"/>
@@ -1104,7 +1113,7 @@
       <c r="A25" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="29"/>
+      <c r="B25" s="33"/>
       <c r="C25" s="22">
         <f>SUM(C20:C24)</f>
         <v>0</v>
@@ -1116,42 +1125,42 @@
       <c r="A26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="30"/>
+      <c r="B26" s="34"/>
       <c r="C26" s="25"/>
       <c r="D26" s="26"/>
       <c r="E26" s="27"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
-      <c r="B27" s="28"/>
+      <c r="B27" s="32"/>
       <c r="C27" s="5"/>
       <c r="D27" s="6"/>
       <c r="E27" s="21"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
-      <c r="B28" s="29"/>
+      <c r="B28" s="33"/>
       <c r="C28" s="8"/>
       <c r="D28" s="9"/>
       <c r="E28" s="8"/>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
-      <c r="B29" s="29"/>
+      <c r="B29" s="33"/>
       <c r="C29" s="8"/>
       <c r="D29" s="9"/>
       <c r="E29" s="8"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
-      <c r="B30" s="29"/>
+      <c r="B30" s="33"/>
       <c r="C30" s="8"/>
       <c r="D30" s="9"/>
       <c r="E30" s="8"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
-      <c r="B31" s="29"/>
+      <c r="B31" s="33"/>
       <c r="C31" s="10"/>
       <c r="D31" s="11"/>
       <c r="E31" s="10"/>
@@ -1160,7 +1169,7 @@
       <c r="A32" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B32" s="29"/>
+      <c r="B32" s="33"/>
       <c r="C32" s="22">
         <f>SUM(C27:C31)</f>
         <v>0</v>
@@ -1172,42 +1181,42 @@
       <c r="A33" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="30"/>
+      <c r="B33" s="34"/>
       <c r="C33" s="25"/>
       <c r="D33" s="26"/>
       <c r="E33" s="27"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
-      <c r="B34" s="28"/>
+      <c r="B34" s="32"/>
       <c r="C34" s="5"/>
       <c r="D34" s="6"/>
       <c r="E34" s="21"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7"/>
-      <c r="B35" s="29"/>
+      <c r="B35" s="33"/>
       <c r="C35" s="8"/>
       <c r="D35" s="9"/>
       <c r="E35" s="8"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="29"/>
+      <c r="B36" s="33"/>
       <c r="C36" s="8"/>
       <c r="D36" s="9"/>
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="29"/>
+      <c r="B37" s="33"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="29"/>
+      <c r="B38" s="33"/>
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
@@ -1216,7 +1225,7 @@
       <c r="A39" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B39" s="29"/>
+      <c r="B39" s="33"/>
       <c r="C39" s="22">
         <f>SUM(C34:C38)</f>
         <v>0</v>
@@ -1228,42 +1237,42 @@
       <c r="A40" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="30"/>
+      <c r="B40" s="34"/>
       <c r="C40" s="25"/>
       <c r="D40" s="26"/>
       <c r="E40" s="27"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
-      <c r="B41" s="28"/>
+      <c r="B41" s="32"/>
       <c r="C41" s="5"/>
       <c r="D41" s="6"/>
       <c r="E41" s="21"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="7"/>
-      <c r="B42" s="29"/>
+      <c r="B42" s="33"/>
       <c r="C42" s="8"/>
       <c r="D42" s="9"/>
       <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="29"/>
+      <c r="B43" s="33"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
-      <c r="B44" s="29"/>
+      <c r="B44" s="33"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10"/>
-      <c r="B45" s="29"/>
+      <c r="B45" s="33"/>
       <c r="C45" s="10"/>
       <c r="D45" s="11"/>
       <c r="E45" s="10"/>
@@ -1272,7 +1281,7 @@
       <c r="A46" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B46" s="29"/>
+      <c r="B46" s="33"/>
       <c r="C46" s="22">
         <f>SUM(C41:C45)</f>
         <v>0</v>
@@ -1284,42 +1293,42 @@
       <c r="A47" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="30"/>
+      <c r="B47" s="34"/>
       <c r="C47" s="25"/>
       <c r="D47" s="26"/>
       <c r="E47" s="27"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="4"/>
-      <c r="B48" s="28"/>
+      <c r="B48" s="32"/>
       <c r="C48" s="5"/>
       <c r="D48" s="6"/>
       <c r="E48" s="21"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="29"/>
+      <c r="B49" s="33"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="29"/>
+      <c r="B50" s="33"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="29"/>
+      <c r="B51" s="33"/>
       <c r="C51" s="8"/>
       <c r="D51" s="9"/>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
-      <c r="B52" s="29"/>
+      <c r="B52" s="33"/>
       <c r="C52" s="10"/>
       <c r="D52" s="11"/>
       <c r="E52" s="10"/>
@@ -1328,7 +1337,7 @@
       <c r="A53" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B53" s="29"/>
+      <c r="B53" s="33"/>
       <c r="C53" s="22">
         <f>SUM(C48:C52)</f>
         <v>0</v>
@@ -1340,42 +1349,42 @@
       <c r="A54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="30"/>
+      <c r="B54" s="34"/>
       <c r="C54" s="25"/>
       <c r="D54" s="26"/>
       <c r="E54" s="27"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4"/>
-      <c r="B55" s="28"/>
+      <c r="B55" s="32"/>
       <c r="C55" s="5"/>
       <c r="D55" s="6"/>
       <c r="E55" s="21"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="29"/>
+      <c r="B56" s="33"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="29"/>
+      <c r="B57" s="33"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="29"/>
+      <c r="B58" s="33"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
-      <c r="B59" s="29"/>
+      <c r="B59" s="33"/>
       <c r="C59" s="10"/>
       <c r="D59" s="11"/>
       <c r="E59" s="10"/>
@@ -1384,7 +1393,7 @@
       <c r="A60" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B60" s="29"/>
+      <c r="B60" s="33"/>
       <c r="C60" s="22">
         <f>SUM(C55:C59)</f>
         <v>0</v>
@@ -1396,42 +1405,42 @@
       <c r="A61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="30"/>
+      <c r="B61" s="34"/>
       <c r="C61" s="25"/>
       <c r="D61" s="26"/>
       <c r="E61" s="27"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4"/>
-      <c r="B62" s="28"/>
+      <c r="B62" s="32"/>
       <c r="C62" s="5"/>
       <c r="D62" s="6"/>
       <c r="E62" s="21"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="29"/>
+      <c r="B63" s="33"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="29"/>
+      <c r="B64" s="33"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="29"/>
+      <c r="B65" s="33"/>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="29"/>
+      <c r="B66" s="33"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -1440,7 +1449,7 @@
       <c r="A67" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B67" s="29"/>
+      <c r="B67" s="33"/>
       <c r="C67" s="22">
         <f>SUM(C62:C66)</f>
         <v>0</v>
@@ -1452,42 +1461,42 @@
       <c r="A68" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="30"/>
+      <c r="B68" s="34"/>
       <c r="C68" s="25"/>
       <c r="D68" s="26"/>
       <c r="E68" s="27"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="4"/>
-      <c r="B69" s="28"/>
+      <c r="B69" s="32"/>
       <c r="C69" s="5"/>
       <c r="D69" s="6"/>
       <c r="E69" s="21"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="29"/>
+      <c r="B70" s="33"/>
       <c r="C70" s="8"/>
       <c r="D70" s="9"/>
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="29"/>
+      <c r="B71" s="33"/>
       <c r="C71" s="8"/>
       <c r="D71" s="9"/>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
-      <c r="B72" s="29"/>
+      <c r="B72" s="33"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="10"/>
-      <c r="B73" s="29"/>
+      <c r="B73" s="33"/>
       <c r="C73" s="10"/>
       <c r="D73" s="11"/>
       <c r="E73" s="10"/>
@@ -1496,7 +1505,7 @@
       <c r="A74" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B74" s="29"/>
+      <c r="B74" s="33"/>
       <c r="C74" s="22">
         <f>SUM(C69:C73)</f>
         <v>0</v>
@@ -1508,7 +1517,7 @@
       <c r="A75" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="30"/>
+      <c r="B75" s="34"/>
       <c r="C75" s="25"/>
       <c r="D75" s="26"/>
       <c r="E75" s="27"/>
@@ -1517,35 +1526,35 @@
       <c r="A76" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="28"/>
+      <c r="B76" s="32"/>
       <c r="C76" s="5"/>
       <c r="D76" s="6"/>
       <c r="E76" s="21"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="29"/>
+      <c r="B77" s="33"/>
       <c r="C77" s="8"/>
       <c r="D77" s="9"/>
       <c r="E77" s="8"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7"/>
-      <c r="B78" s="29"/>
+      <c r="B78" s="33"/>
       <c r="C78" s="8"/>
       <c r="D78" s="9"/>
       <c r="E78" s="8"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
-      <c r="B79" s="29"/>
+      <c r="B79" s="33"/>
       <c r="C79" s="8"/>
       <c r="D79" s="9"/>
       <c r="E79" s="8"/>
     </row>
     <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10"/>
-      <c r="B80" s="29"/>
+      <c r="B80" s="33"/>
       <c r="C80" s="10"/>
       <c r="D80" s="11"/>
       <c r="E80" s="10"/>
@@ -1554,7 +1563,7 @@
       <c r="A81" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B81" s="29"/>
+      <c r="B81" s="33"/>
       <c r="C81" s="22">
         <f>SUM(C76:C80)</f>
         <v>0</v>
@@ -1566,42 +1575,42 @@
       <c r="A82" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B82" s="30"/>
+      <c r="B82" s="34"/>
       <c r="C82" s="25"/>
       <c r="D82" s="26"/>
       <c r="E82" s="27"/>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="4"/>
-      <c r="B83" s="28"/>
+      <c r="B83" s="32"/>
       <c r="C83" s="5"/>
       <c r="D83" s="6"/>
       <c r="E83" s="21"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
-      <c r="B84" s="29"/>
+      <c r="B84" s="33"/>
       <c r="C84" s="8"/>
       <c r="D84" s="9"/>
       <c r="E84" s="8"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="29"/>
+      <c r="B85" s="33"/>
       <c r="C85" s="8"/>
       <c r="D85" s="9"/>
       <c r="E85" s="8"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="29"/>
+      <c r="B86" s="33"/>
       <c r="C86" s="8"/>
       <c r="D86" s="9"/>
       <c r="E86" s="8"/>
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="29"/>
+      <c r="B87" s="33"/>
       <c r="C87" s="10"/>
       <c r="D87" s="11"/>
       <c r="E87" s="10"/>
@@ -1610,7 +1619,7 @@
       <c r="A88" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B88" s="29"/>
+      <c r="B88" s="33"/>
       <c r="C88" s="22">
         <f>SUM(C83:C87)</f>
         <v>0</v>
@@ -1622,19 +1631,19 @@
       <c r="A89" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B89" s="30"/>
+      <c r="B89" s="34"/>
       <c r="C89" s="25"/>
       <c r="D89" s="26"/>
       <c r="E89" s="27"/>
     </row>
     <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="31" t="s">
+      <c r="A90" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="B90" s="32"/>
+      <c r="B90" s="36"/>
       <c r="C90" s="13">
         <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>3</v>
+        <v>4.6000000000000005</v>
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="15"/>
@@ -1649,6 +1658,31 @@
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="C89:E89"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B69:B75"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="B27:B33"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="B34:B40"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="B48:B54"/>
+    <mergeCell ref="B55:B61"/>
+    <mergeCell ref="B62:B68"/>
+    <mergeCell ref="B76:B82"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="B1:C1"/>
@@ -1665,31 +1699,6 @@
     <mergeCell ref="B20:B26"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="C26:E26"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="B34:B40"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="B76:B82"/>
-    <mergeCell ref="B27:B33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="B69:B75"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="C89:E89"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C83:C88 B13 C13:C18 B20 C20:C25 B27 C27:C32 B34 C34:C39 B41 C41:C46 B48 C48:C53 B55 C55:C60 B62 C62:C67 B69 C69:C74 B76 C76:C81 B83 C7:C11" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1708,6 +1717,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -1869,12 +1884,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1885,6 +1894,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1902,15 +1920,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat(app): avancée des différentes fonctionnalitées demandées pour le premier rendu. PlacerTour, DeplacerEnnemis, TirerTour, CalculerDegats
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6E1F62A-9799-42D4-9C7B-35B8179E7C00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B5E42BF-20BC-41F5-BDBD-F33E3619CCDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5445" yWindow="1905" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$90</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$73</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="48">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -148,10 +148,52 @@
     <t>Visual Studio</t>
   </si>
   <si>
-    <t>Création du fichier et début de la rédaction du code</t>
-  </si>
-  <si>
     <t>Création et début de rédaction des méthodes pour le choix de tours et déplacement d'ennemi</t>
+  </si>
+  <si>
+    <t>Création de tout les éléments nécessaires à la création du projet</t>
+  </si>
+  <si>
+    <t>Commencement de la rédaction du code avec les fonctions de choix de placement des tours + déplacement des ennemis</t>
+  </si>
+  <si>
+    <t>Création du fichier Vscode et réflexion sur la manière d'aborder les premières fonctions</t>
+  </si>
+  <si>
+    <t>Finir d'implémenter la fonctionnalité de déplacement des tours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">continuer le déplacement d'un ennemi avec plusieurs essais et complication  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avancée dans la rédaction des deux premières fonctions du code </t>
+  </si>
+  <si>
+    <t>Avancée dans la rédaction des fonctions DeplacerEnnemis et TirerTour</t>
+  </si>
+  <si>
+    <t>Finir d'implémenter la fonctionnalité qui permet le déplacement d'un ennemi</t>
+  </si>
+  <si>
+    <t>début de rédaction de la méthode servant à tirer sur les ennemis avec les tours</t>
+  </si>
+  <si>
+    <t>Finir d'implémenter la fonctionnalité qui permet au tour de tirer sur les ennemis</t>
+  </si>
+  <si>
+    <t>En parallèle faire la dernière fonctionnalité servant à compter les dégats " CalculerDegats "</t>
+  </si>
+  <si>
+    <t>Finir d'implémenter la fonctionnalité qui permet de calculer les dégats infligés aux ennemis</t>
+  </si>
+  <si>
+    <t>Avancée dans la rédaction des fonctions TirerTour et CalculerDegats</t>
+  </si>
+  <si>
+    <t>Avancée dans la rédaction des fonctions CalculerDegats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit réalisé </t>
   </si>
 </sst>
 </file>
@@ -496,18 +538,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -525,6 +555,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -842,13 +884,13 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="80.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="91.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="36" style="1" customWidth="1"/>
@@ -859,10 +901,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="28"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -872,10 +914,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -887,10 +929,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="28"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -902,12 +944,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -930,7 +972,9 @@
       <c r="A6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="32"/>
+      <c r="B6" s="28">
+        <v>45671</v>
+      </c>
       <c r="C6" s="5">
         <v>3</v>
       </c>
@@ -943,7 +987,7 @@
       <c r="A7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -956,7 +1000,7 @@
       <c r="A8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="33"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="8">
         <v>3</v>
       </c>
@@ -969,7 +1013,7 @@
       <c r="A9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="33"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="8">
         <v>1</v>
       </c>
@@ -982,20 +1026,22 @@
       <c r="A10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="33"/>
+      <c r="B10" s="29"/>
       <c r="C10" s="10">
         <v>2</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" s="10"/>
+        <v>35</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1007,59 +1053,88 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="34"/>
-      <c r="C12" s="25"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="25" t="s">
+        <v>33</v>
+      </c>
       <c r="D12" s="26"/>
       <c r="E12" s="27"/>
     </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="32"/>
+      <c r="B13" s="28">
+        <v>45678</v>
+      </c>
       <c r="C13" s="5">
         <v>6</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="21"/>
-    </row>
-    <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="33"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="8"/>
-    </row>
-    <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="33"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="8"/>
+        <v>32</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="29"/>
+      <c r="C14" s="22">
+        <f>SUM(C13:C13)</f>
+        <v>6</v>
+      </c>
+      <c r="D14" s="23"/>
+      <c r="E14" s="24"/>
+    </row>
+    <row r="15" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="30"/>
+      <c r="C15" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="33"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="8"/>
+      <c r="A16" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="28">
+        <v>45681</v>
+      </c>
+      <c r="C16" s="5">
+        <v>4</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E16" s="21"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="10"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="10"/>
+      <c r="A17" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="29"/>
+      <c r="C17" s="8">
+        <v>2</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="33"/>
+      <c r="B18" s="29"/>
       <c r="C18" s="22">
-        <f>SUM(C13:C17)</f>
+        <f>SUM(C16:C17)</f>
         <v>6</v>
       </c>
       <c r="D18" s="23"/>
@@ -1069,645 +1144,563 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="34"/>
-      <c r="C19" s="25"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="25" t="s">
+        <v>38</v>
+      </c>
       <c r="D19" s="26"/>
       <c r="E19" s="27"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="4"/>
-      <c r="B20" s="32"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="6"/>
+      <c r="A20" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="28">
+        <v>45682</v>
+      </c>
+      <c r="C20" s="5">
+        <v>4</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>40</v>
+      </c>
       <c r="E20" s="21"/>
     </row>
-    <row r="21" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="33"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="9"/>
+    <row r="21" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21" s="29"/>
+      <c r="C21" s="8">
+        <v>2</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>41</v>
+      </c>
       <c r="E21" s="8"/>
     </row>
-    <row r="22" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="8"/>
-    </row>
-    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="8"/>
-    </row>
-    <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="10"/>
-      <c r="B24" s="33"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="10"/>
+    <row r="22" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="29"/>
+      <c r="C22" s="22">
+        <f>SUM(C20:C21)</f>
+        <v>6</v>
+      </c>
+      <c r="D22" s="23"/>
+      <c r="E22" s="24"/>
+    </row>
+    <row r="23" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" s="30"/>
+      <c r="C23" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" s="26"/>
+      <c r="E23" s="27"/>
+    </row>
+    <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="28">
+        <v>46048</v>
+      </c>
+      <c r="C24" s="5">
+        <v>2</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E24" s="21"/>
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" s="33"/>
-      <c r="C25" s="22">
-        <f>SUM(C20:C24)</f>
-        <v>0</v>
-      </c>
-      <c r="D25" s="23"/>
-      <c r="E25" s="24"/>
+      <c r="A25" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="29"/>
+      <c r="C25" s="8">
+        <v>2</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="29"/>
+      <c r="C26" s="22">
+        <f>SUM(C24:C25)</f>
+        <v>4</v>
+      </c>
+      <c r="D26" s="23"/>
+      <c r="E26" s="24"/>
+    </row>
+    <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="34"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="27"/>
-    </row>
-    <row r="27" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="4"/>
-      <c r="B27" s="32"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="21"/>
-    </row>
-    <row r="28" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="7"/>
-      <c r="B28" s="33"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="8"/>
-    </row>
-    <row r="29" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="7"/>
-      <c r="B29" s="33"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="8"/>
-    </row>
-    <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="7"/>
-      <c r="B30" s="33"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="8"/>
-    </row>
-    <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="10"/>
-      <c r="B31" s="33"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="10"/>
-    </row>
-    <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
+      <c r="B27" s="30"/>
+      <c r="C27" s="25" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="26"/>
+      <c r="E27" s="27"/>
+    </row>
+    <row r="28" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" s="28">
+        <v>46049</v>
+      </c>
+      <c r="C28" s="5">
+        <v>2</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="21"/>
+    </row>
+    <row r="29" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B32" s="33"/>
-      <c r="C32" s="22">
-        <f>SUM(C27:C31)</f>
+      <c r="B29" s="29"/>
+      <c r="C29" s="22">
+        <f>SUM(C28:C28)</f>
+        <v>2</v>
+      </c>
+      <c r="D29" s="23"/>
+      <c r="E29" s="24"/>
+    </row>
+    <row r="30" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B30" s="30"/>
+      <c r="C30" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" s="26"/>
+      <c r="E30" s="27"/>
+    </row>
+    <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="4"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="21"/>
+    </row>
+    <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="7"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="8"/>
+    </row>
+    <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="7"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="8"/>
+    </row>
+    <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="7"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="8"/>
+    </row>
+    <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="10"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="10"/>
+    </row>
+    <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" s="29"/>
+      <c r="C36" s="22">
+        <f>SUM(C31:C35)</f>
         <v>0</v>
       </c>
-      <c r="D32" s="23"/>
-      <c r="E32" s="24"/>
-    </row>
-    <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="12" t="s">
+      <c r="D36" s="23"/>
+      <c r="E36" s="24"/>
+    </row>
+    <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="26"/>
-      <c r="E33" s="27"/>
-    </row>
-    <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="6"/>
-      <c r="E34" s="21"/>
-    </row>
-    <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="7"/>
-      <c r="B35" s="33"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="9"/>
-      <c r="E35" s="8"/>
-    </row>
-    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="8"/>
-    </row>
-    <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="7"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="8"/>
-    </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="10"/>
-      <c r="B38" s="33"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="10"/>
-    </row>
-    <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="12" t="s">
+      <c r="B37" s="30"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="27"/>
+    </row>
+    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="4"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="6"/>
+      <c r="E38" s="21"/>
+    </row>
+    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="7"/>
+      <c r="B39" s="29"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="8"/>
+    </row>
+    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="7"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="8"/>
+    </row>
+    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="7"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="8"/>
+    </row>
+    <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="10"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="11"/>
+      <c r="E42" s="10"/>
+    </row>
+    <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B39" s="33"/>
-      <c r="C39" s="22">
-        <f>SUM(C34:C38)</f>
+      <c r="B43" s="29"/>
+      <c r="C43" s="22">
+        <f>SUM(C38:C42)</f>
         <v>0</v>
       </c>
-      <c r="D39" s="23"/>
-      <c r="E39" s="24"/>
-    </row>
-    <row r="40" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
+      <c r="D43" s="23"/>
+      <c r="E43" s="24"/>
+    </row>
+    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="34"/>
-      <c r="C40" s="25"/>
-      <c r="D40" s="26"/>
-      <c r="E40" s="27"/>
-    </row>
-    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="4"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="6"/>
-      <c r="E41" s="21"/>
-    </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="7"/>
-      <c r="B42" s="33"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="8"/>
-    </row>
-    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="7"/>
-      <c r="B43" s="33"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="8"/>
-    </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="7"/>
-      <c r="B44" s="33"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="8"/>
-    </row>
-    <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="10"/>
-      <c r="B45" s="33"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="11"/>
-      <c r="E45" s="10"/>
-    </row>
-    <row r="46" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="12" t="s">
+      <c r="B44" s="30"/>
+      <c r="C44" s="25"/>
+      <c r="D44" s="26"/>
+      <c r="E44" s="27"/>
+    </row>
+    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="4"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="5"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="21"/>
+    </row>
+    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="7"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="8"/>
+    </row>
+    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="7"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="8"/>
+    </row>
+    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="7"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="10"/>
+      <c r="B49" s="29"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="11"/>
+      <c r="E49" s="10"/>
+    </row>
+    <row r="50" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B46" s="33"/>
-      <c r="C46" s="22">
-        <f>SUM(C41:C45)</f>
+      <c r="B50" s="29"/>
+      <c r="C50" s="22">
+        <f>SUM(C45:C49)</f>
         <v>0</v>
       </c>
-      <c r="D46" s="23"/>
-      <c r="E46" s="24"/>
-    </row>
-    <row r="47" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="12" t="s">
+      <c r="D50" s="23"/>
+      <c r="E50" s="24"/>
+    </row>
+    <row r="51" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="34"/>
-      <c r="C47" s="25"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="27"/>
-    </row>
-    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="4"/>
-      <c r="B48" s="32"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="21"/>
-    </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="7"/>
-      <c r="B49" s="33"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="9"/>
-      <c r="E49" s="8"/>
-    </row>
-    <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="7"/>
-      <c r="B50" s="33"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="8"/>
-    </row>
-    <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="7"/>
-      <c r="B51" s="33"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="8"/>
-    </row>
-    <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="10"/>
-      <c r="B52" s="33"/>
-      <c r="C52" s="10"/>
-      <c r="D52" s="11"/>
-      <c r="E52" s="10"/>
-    </row>
-    <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="12" t="s">
+      <c r="B51" s="30"/>
+      <c r="C51" s="25"/>
+      <c r="D51" s="26"/>
+      <c r="E51" s="27"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="4"/>
+      <c r="B52" s="28"/>
+      <c r="C52" s="5"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="21"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="7"/>
+      <c r="B53" s="29"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="8"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="7"/>
+      <c r="B54" s="29"/>
+      <c r="C54" s="8"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="8"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="7"/>
+      <c r="B55" s="29"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="8"/>
+    </row>
+    <row r="56" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="10"/>
+      <c r="B56" s="29"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="10"/>
+    </row>
+    <row r="57" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B53" s="33"/>
-      <c r="C53" s="22">
-        <f>SUM(C48:C52)</f>
+      <c r="B57" s="29"/>
+      <c r="C57" s="22">
+        <f>SUM(C52:C56)</f>
         <v>0</v>
       </c>
-      <c r="D53" s="23"/>
-      <c r="E53" s="24"/>
-    </row>
-    <row r="54" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="12" t="s">
+      <c r="D57" s="23"/>
+      <c r="E57" s="24"/>
+    </row>
+    <row r="58" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="34"/>
-      <c r="C54" s="25"/>
-      <c r="D54" s="26"/>
-      <c r="E54" s="27"/>
-    </row>
-    <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="4"/>
-      <c r="B55" s="32"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="6"/>
-      <c r="E55" s="21"/>
-    </row>
-    <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="7"/>
-      <c r="B56" s="33"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="9"/>
-      <c r="E56" s="8"/>
-    </row>
-    <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="7"/>
-      <c r="B57" s="33"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="8"/>
-    </row>
-    <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="7"/>
-      <c r="B58" s="33"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="8"/>
-    </row>
-    <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="10"/>
-      <c r="B59" s="33"/>
-      <c r="C59" s="10"/>
-      <c r="D59" s="11"/>
-      <c r="E59" s="10"/>
-    </row>
-    <row r="60" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="12" t="s">
+      <c r="B58" s="30"/>
+      <c r="C58" s="25"/>
+      <c r="D58" s="26"/>
+      <c r="E58" s="27"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B59" s="28"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="21"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="7"/>
+      <c r="B60" s="29"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="8"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="7"/>
+      <c r="B61" s="29"/>
+      <c r="C61" s="8"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="8"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="7"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="9"/>
+      <c r="E62" s="8"/>
+    </row>
+    <row r="63" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="10"/>
+      <c r="B63" s="29"/>
+      <c r="C63" s="10"/>
+      <c r="D63" s="11"/>
+      <c r="E63" s="10"/>
+    </row>
+    <row r="64" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B60" s="33"/>
-      <c r="C60" s="22">
-        <f>SUM(C55:C59)</f>
+      <c r="B64" s="29"/>
+      <c r="C64" s="22">
+        <f>SUM(C59:C63)</f>
         <v>0</v>
       </c>
-      <c r="D60" s="23"/>
-      <c r="E60" s="24"/>
-    </row>
-    <row r="61" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="12" t="s">
+      <c r="D64" s="23"/>
+      <c r="E64" s="24"/>
+    </row>
+    <row r="65" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="34"/>
-      <c r="C61" s="25"/>
-      <c r="D61" s="26"/>
-      <c r="E61" s="27"/>
-    </row>
-    <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="4"/>
-      <c r="B62" s="32"/>
-      <c r="C62" s="5"/>
-      <c r="D62" s="6"/>
-      <c r="E62" s="21"/>
-    </row>
-    <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="7"/>
-      <c r="B63" s="33"/>
-      <c r="C63" s="8"/>
-      <c r="D63" s="9"/>
-      <c r="E63" s="8"/>
-    </row>
-    <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="7"/>
-      <c r="B64" s="33"/>
-      <c r="C64" s="8"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="8"/>
-    </row>
-    <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="7"/>
-      <c r="B65" s="33"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="8"/>
-    </row>
-    <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="10"/>
-      <c r="B66" s="33"/>
-      <c r="C66" s="10"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="10"/>
-    </row>
-    <row r="67" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="12" t="s">
+      <c r="B65" s="30"/>
+      <c r="C65" s="25"/>
+      <c r="D65" s="26"/>
+      <c r="E65" s="27"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="4"/>
+      <c r="B66" s="28"/>
+      <c r="C66" s="5"/>
+      <c r="D66" s="6"/>
+      <c r="E66" s="21"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="7"/>
+      <c r="B67" s="29"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="8"/>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="7"/>
+      <c r="B68" s="29"/>
+      <c r="C68" s="8"/>
+      <c r="D68" s="9"/>
+      <c r="E68" s="8"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="7"/>
+      <c r="B69" s="29"/>
+      <c r="C69" s="8"/>
+      <c r="D69" s="9"/>
+      <c r="E69" s="8"/>
+    </row>
+    <row r="70" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="10"/>
+      <c r="B70" s="29"/>
+      <c r="C70" s="10"/>
+      <c r="D70" s="11"/>
+      <c r="E70" s="10"/>
+    </row>
+    <row r="71" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B67" s="33"/>
-      <c r="C67" s="22">
-        <f>SUM(C62:C66)</f>
+      <c r="B71" s="29"/>
+      <c r="C71" s="22">
+        <f>SUM(C66:C70)</f>
         <v>0</v>
       </c>
-      <c r="D67" s="23"/>
-      <c r="E67" s="24"/>
-    </row>
-    <row r="68" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="12" t="s">
+      <c r="D71" s="23"/>
+      <c r="E71" s="24"/>
+    </row>
+    <row r="72" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="34"/>
-      <c r="C68" s="25"/>
-      <c r="D68" s="26"/>
-      <c r="E68" s="27"/>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="4"/>
-      <c r="B69" s="32"/>
-      <c r="C69" s="5"/>
-      <c r="D69" s="6"/>
-      <c r="E69" s="21"/>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="7"/>
-      <c r="B70" s="33"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="9"/>
-      <c r="E70" s="8"/>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="7"/>
-      <c r="B71" s="33"/>
-      <c r="C71" s="8"/>
-      <c r="D71" s="9"/>
-      <c r="E71" s="8"/>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="7"/>
-      <c r="B72" s="33"/>
-      <c r="C72" s="8"/>
-      <c r="D72" s="9"/>
-      <c r="E72" s="8"/>
-    </row>
-    <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="10"/>
-      <c r="B73" s="33"/>
-      <c r="C73" s="10"/>
-      <c r="D73" s="11"/>
-      <c r="E73" s="10"/>
-    </row>
-    <row r="74" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B74" s="33"/>
-      <c r="C74" s="22">
-        <f>SUM(C69:C73)</f>
-        <v>0</v>
-      </c>
-      <c r="D74" s="23"/>
-      <c r="E74" s="24"/>
-    </row>
-    <row r="75" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B75" s="34"/>
-      <c r="C75" s="25"/>
-      <c r="D75" s="26"/>
-      <c r="E75" s="27"/>
+      <c r="B72" s="30"/>
+      <c r="C72" s="25"/>
+      <c r="D72" s="26"/>
+      <c r="E72" s="27"/>
+    </row>
+    <row r="73" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="B73" s="32"/>
+      <c r="C73" s="13">
+        <f>MROUND(SUM(C6:C72) /8,0.2)</f>
+        <v>9</v>
+      </c>
+      <c r="D73" s="14"/>
+      <c r="E73" s="15"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="16" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B76" s="32"/>
-      <c r="C76" s="5"/>
-      <c r="D76" s="6"/>
-      <c r="E76" s="21"/>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="7"/>
-      <c r="B77" s="33"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="9"/>
-      <c r="E77" s="8"/>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="7"/>
-      <c r="B78" s="33"/>
-      <c r="C78" s="8"/>
-      <c r="D78" s="9"/>
-      <c r="E78" s="8"/>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="7"/>
-      <c r="B79" s="33"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="9"/>
-      <c r="E79" s="8"/>
-    </row>
-    <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="10"/>
-      <c r="B80" s="33"/>
-      <c r="C80" s="10"/>
-      <c r="D80" s="11"/>
-      <c r="E80" s="10"/>
-    </row>
-    <row r="81" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B81" s="33"/>
-      <c r="C81" s="22">
-        <f>SUM(C76:C80)</f>
-        <v>0</v>
-      </c>
-      <c r="D81" s="23"/>
-      <c r="E81" s="24"/>
-    </row>
-    <row r="82" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B82" s="34"/>
-      <c r="C82" s="25"/>
-      <c r="D82" s="26"/>
-      <c r="E82" s="27"/>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="4"/>
-      <c r="B83" s="32"/>
-      <c r="C83" s="5"/>
-      <c r="D83" s="6"/>
-      <c r="E83" s="21"/>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="7"/>
-      <c r="B84" s="33"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="9"/>
-      <c r="E84" s="8"/>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="7"/>
-      <c r="B85" s="33"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="9"/>
-      <c r="E85" s="8"/>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" s="7"/>
-      <c r="B86" s="33"/>
-      <c r="C86" s="8"/>
-      <c r="D86" s="9"/>
-      <c r="E86" s="8"/>
-    </row>
-    <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="10"/>
-      <c r="B87" s="33"/>
-      <c r="C87" s="10"/>
-      <c r="D87" s="11"/>
-      <c r="E87" s="10"/>
-    </row>
-    <row r="88" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B88" s="33"/>
-      <c r="C88" s="22">
-        <f>SUM(C83:C87)</f>
-        <v>0</v>
-      </c>
-      <c r="D88" s="23"/>
-      <c r="E88" s="24"/>
-    </row>
-    <row r="89" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B89" s="34"/>
-      <c r="C89" s="25"/>
-      <c r="D89" s="26"/>
-      <c r="E89" s="27"/>
-    </row>
-    <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="35" t="s">
-        <v>14</v>
-      </c>
-      <c r="B90" s="36"/>
-      <c r="C90" s="13">
-        <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>4.6000000000000005</v>
-      </c>
-      <c r="D90" s="14"/>
-      <c r="E90" s="15"/>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="16"/>
+      <c r="A76" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="C89:E89"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="B69:B75"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="B27:B33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="B34:B40"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="B76:B82"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="C44:E44"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="C37:E37"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="B6:B12"/>
-    <mergeCell ref="B13:B19"/>
+    <mergeCell ref="B13:B15"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="B16:B19"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="C19:E19"/>
-    <mergeCell ref="B20:B26"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B37"/>
+    <mergeCell ref="B38:B44"/>
+    <mergeCell ref="B45:B51"/>
+    <mergeCell ref="B59:B65"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="B52:B58"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="B66:B72"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="C72:E72"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C83:C88 B13 C13:C18 B20 C20:C25 B27 C27:C32 B34 C34:C39 B41 C41:C46 B48 C48:C53 B55 C55:C60 B62 C62:C67 B69 C69:C74 B76 C76:C81 B83 C7:C11" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C66:C71 B13 B16 B20 B24 B28 B31 C31:C36 B38 C38:C43 B45 C45:C50 B52 C52:C57 B59 C59:C64 B66 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="46" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="43" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Etml_font,Normal"&amp;22ETML&amp;R&amp;G</oddHeader>
     <oddFooter>&amp;L&amp;14&amp;D&amp;R&amp;14Journal</oddFooter>
@@ -1717,12 +1710,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -1884,6 +1871,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1894,15 +1887,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1920,6 +1904,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat(suitev1): commencement de nouvelles fonctionnalités et corrections de nouveaux bugs rencontrés
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B5E42BF-20BC-41F5-BDBD-F33E3619CCDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B047783D-5BBA-4ADC-BFED-A86340BF2EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5445" yWindow="1905" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5985" yWindow="1710" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="50">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -194,6 +194,12 @@
   </si>
   <si>
     <t xml:space="preserve">Commit réalisé </t>
+  </si>
+  <si>
+    <t>Validation des dernières modifs pour la v1 + rendu v1</t>
+  </si>
+  <si>
+    <t>Avancée de nouvelles choses et corrections de nouveaux bugs rencontrés</t>
   </si>
 </sst>
 </file>
@@ -538,6 +544,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -555,18 +573,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -901,10 +907,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="33"/>
+      <c r="C1" s="28"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -914,10 +920,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="28"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -929,10 +935,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="28"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -944,12 +950,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -972,7 +978,7 @@
       <c r="A6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="28">
+      <c r="B6" s="32">
         <v>45671</v>
       </c>
       <c r="C6" s="5">
@@ -987,7 +993,7 @@
       <c r="A7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="33"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -1000,7 +1006,7 @@
       <c r="A8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="33"/>
       <c r="C8" s="8">
         <v>3</v>
       </c>
@@ -1013,7 +1019,7 @@
       <c r="A9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="33"/>
       <c r="C9" s="8">
         <v>1</v>
       </c>
@@ -1026,7 +1032,7 @@
       <c r="A10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="29"/>
+      <c r="B10" s="33"/>
       <c r="C10" s="10">
         <v>2</v>
       </c>
@@ -1041,7 +1047,7 @@
       <c r="A11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="29"/>
+      <c r="B11" s="33"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1053,7 +1059,7 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="30"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="25" t="s">
         <v>33</v>
       </c>
@@ -1064,7 +1070,7 @@
       <c r="A13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="32">
         <v>45678</v>
       </c>
       <c r="C13" s="5">
@@ -1081,7 +1087,7 @@
       <c r="A14" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="29"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="22">
         <f>SUM(C13:C13)</f>
         <v>6</v>
@@ -1093,7 +1099,7 @@
       <c r="A15" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="30"/>
+      <c r="B15" s="34"/>
       <c r="C15" s="25" t="s">
         <v>34</v>
       </c>
@@ -1104,7 +1110,7 @@
       <c r="A16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="28">
+      <c r="B16" s="32">
         <v>45681</v>
       </c>
       <c r="C16" s="5">
@@ -1119,7 +1125,7 @@
       <c r="A17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="29"/>
+      <c r="B17" s="33"/>
       <c r="C17" s="8">
         <v>2</v>
       </c>
@@ -1132,7 +1138,7 @@
       <c r="A18" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="29"/>
+      <c r="B18" s="33"/>
       <c r="C18" s="22">
         <f>SUM(C16:C17)</f>
         <v>6</v>
@@ -1144,7 +1150,7 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="30"/>
+      <c r="B19" s="34"/>
       <c r="C19" s="25" t="s">
         <v>38</v>
       </c>
@@ -1155,7 +1161,7 @@
       <c r="A20" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="28">
+      <c r="B20" s="32">
         <v>45682</v>
       </c>
       <c r="C20" s="5">
@@ -1170,7 +1176,7 @@
       <c r="A21" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="29"/>
+      <c r="B21" s="33"/>
       <c r="C21" s="8">
         <v>2</v>
       </c>
@@ -1183,7 +1189,7 @@
       <c r="A22" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="29"/>
+      <c r="B22" s="33"/>
       <c r="C22" s="22">
         <f>SUM(C20:C21)</f>
         <v>6</v>
@@ -1195,7 +1201,7 @@
       <c r="A23" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="30"/>
+      <c r="B23" s="34"/>
       <c r="C23" s="25" t="s">
         <v>39</v>
       </c>
@@ -1206,7 +1212,7 @@
       <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="28">
+      <c r="B24" s="32">
         <v>46048</v>
       </c>
       <c r="C24" s="5">
@@ -1221,7 +1227,7 @@
       <c r="A25" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="29"/>
+      <c r="B25" s="33"/>
       <c r="C25" s="8">
         <v>2</v>
       </c>
@@ -1234,7 +1240,7 @@
       <c r="A26" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="29"/>
+      <c r="B26" s="33"/>
       <c r="C26" s="22">
         <f>SUM(C24:C25)</f>
         <v>4</v>
@@ -1246,7 +1252,7 @@
       <c r="A27" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B27" s="30"/>
+      <c r="B27" s="34"/>
       <c r="C27" s="25" t="s">
         <v>45</v>
       </c>
@@ -1257,7 +1263,7 @@
       <c r="A28" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="28">
+      <c r="B28" s="32">
         <v>46049</v>
       </c>
       <c r="C28" s="5">
@@ -1272,7 +1278,7 @@
       <c r="A29" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="29"/>
+      <c r="B29" s="33"/>
       <c r="C29" s="22">
         <f>SUM(C28:C28)</f>
         <v>2</v>
@@ -1284,7 +1290,7 @@
       <c r="A30" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="30"/>
+      <c r="B30" s="34"/>
       <c r="C30" s="25" t="s">
         <v>46</v>
       </c>
@@ -1292,36 +1298,52 @@
       <c r="E30" s="27"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="4"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="21"/>
+      <c r="A31" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" s="32"/>
+      <c r="C31" s="5">
+        <v>6</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="7"/>
-      <c r="B32" s="29"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="9"/>
-      <c r="E32" s="8"/>
+      <c r="A32" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B32" s="33"/>
+      <c r="C32" s="8">
+        <v>6</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7"/>
-      <c r="B33" s="29"/>
+      <c r="B33" s="33"/>
       <c r="C33" s="8"/>
       <c r="D33" s="9"/>
       <c r="E33" s="8"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7"/>
-      <c r="B34" s="29"/>
+      <c r="B34" s="33"/>
       <c r="C34" s="8"/>
       <c r="D34" s="9"/>
       <c r="E34" s="8"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="10"/>
-      <c r="B35" s="29"/>
+      <c r="B35" s="33"/>
       <c r="C35" s="10"/>
       <c r="D35" s="11"/>
       <c r="E35" s="10"/>
@@ -1330,10 +1352,10 @@
       <c r="A36" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="29"/>
+      <c r="B36" s="33"/>
       <c r="C36" s="22">
         <f>SUM(C31:C35)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D36" s="23"/>
       <c r="E36" s="24"/>
@@ -1342,42 +1364,42 @@
       <c r="A37" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B37" s="30"/>
+      <c r="B37" s="34"/>
       <c r="C37" s="25"/>
       <c r="D37" s="26"/>
       <c r="E37" s="27"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
-      <c r="B38" s="28"/>
+      <c r="B38" s="32"/>
       <c r="C38" s="5"/>
       <c r="D38" s="6"/>
       <c r="E38" s="21"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="7"/>
-      <c r="B39" s="29"/>
+      <c r="B39" s="33"/>
       <c r="C39" s="8"/>
       <c r="D39" s="9"/>
       <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7"/>
-      <c r="B40" s="29"/>
+      <c r="B40" s="33"/>
       <c r="C40" s="8"/>
       <c r="D40" s="9"/>
       <c r="E40" s="8"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="7"/>
-      <c r="B41" s="29"/>
+      <c r="B41" s="33"/>
       <c r="C41" s="8"/>
       <c r="D41" s="9"/>
       <c r="E41" s="8"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="10"/>
-      <c r="B42" s="29"/>
+      <c r="B42" s="33"/>
       <c r="C42" s="10"/>
       <c r="D42" s="11"/>
       <c r="E42" s="10"/>
@@ -1386,7 +1408,7 @@
       <c r="A43" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B43" s="29"/>
+      <c r="B43" s="33"/>
       <c r="C43" s="22">
         <f>SUM(C38:C42)</f>
         <v>0</v>
@@ -1398,42 +1420,42 @@
       <c r="A44" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B44" s="30"/>
+      <c r="B44" s="34"/>
       <c r="C44" s="25"/>
       <c r="D44" s="26"/>
       <c r="E44" s="27"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="4"/>
-      <c r="B45" s="28"/>
+      <c r="B45" s="32"/>
       <c r="C45" s="5"/>
       <c r="D45" s="6"/>
       <c r="E45" s="21"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7"/>
-      <c r="B46" s="29"/>
+      <c r="B46" s="33"/>
       <c r="C46" s="8"/>
       <c r="D46" s="9"/>
       <c r="E46" s="8"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7"/>
-      <c r="B47" s="29"/>
+      <c r="B47" s="33"/>
       <c r="C47" s="8"/>
       <c r="D47" s="9"/>
       <c r="E47" s="8"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
-      <c r="B48" s="29"/>
+      <c r="B48" s="33"/>
       <c r="C48" s="8"/>
       <c r="D48" s="9"/>
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="10"/>
-      <c r="B49" s="29"/>
+      <c r="B49" s="33"/>
       <c r="C49" s="10"/>
       <c r="D49" s="11"/>
       <c r="E49" s="10"/>
@@ -1442,7 +1464,7 @@
       <c r="A50" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B50" s="29"/>
+      <c r="B50" s="33"/>
       <c r="C50" s="22">
         <f>SUM(C45:C49)</f>
         <v>0</v>
@@ -1454,42 +1476,42 @@
       <c r="A51" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B51" s="30"/>
+      <c r="B51" s="34"/>
       <c r="C51" s="25"/>
       <c r="D51" s="26"/>
       <c r="E51" s="27"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="4"/>
-      <c r="B52" s="28"/>
+      <c r="B52" s="32"/>
       <c r="C52" s="5"/>
       <c r="D52" s="6"/>
       <c r="E52" s="21"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="7"/>
-      <c r="B53" s="29"/>
+      <c r="B53" s="33"/>
       <c r="C53" s="8"/>
       <c r="D53" s="9"/>
       <c r="E53" s="8"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="7"/>
-      <c r="B54" s="29"/>
+      <c r="B54" s="33"/>
       <c r="C54" s="8"/>
       <c r="D54" s="9"/>
       <c r="E54" s="8"/>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="29"/>
+      <c r="B55" s="33"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="10"/>
-      <c r="B56" s="29"/>
+      <c r="B56" s="33"/>
       <c r="C56" s="10"/>
       <c r="D56" s="11"/>
       <c r="E56" s="10"/>
@@ -1498,7 +1520,7 @@
       <c r="A57" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B57" s="29"/>
+      <c r="B57" s="33"/>
       <c r="C57" s="22">
         <f>SUM(C52:C56)</f>
         <v>0</v>
@@ -1510,7 +1532,7 @@
       <c r="A58" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B58" s="30"/>
+      <c r="B58" s="34"/>
       <c r="C58" s="25"/>
       <c r="D58" s="26"/>
       <c r="E58" s="27"/>
@@ -1519,35 +1541,35 @@
       <c r="A59" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B59" s="28"/>
+      <c r="B59" s="32"/>
       <c r="C59" s="5"/>
       <c r="D59" s="6"/>
       <c r="E59" s="21"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="7"/>
-      <c r="B60" s="29"/>
+      <c r="B60" s="33"/>
       <c r="C60" s="8"/>
       <c r="D60" s="9"/>
       <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="29"/>
+      <c r="B61" s="33"/>
       <c r="C61" s="8"/>
       <c r="D61" s="9"/>
       <c r="E61" s="8"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="29"/>
+      <c r="B62" s="33"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="10"/>
-      <c r="B63" s="29"/>
+      <c r="B63" s="33"/>
       <c r="C63" s="10"/>
       <c r="D63" s="11"/>
       <c r="E63" s="10"/>
@@ -1556,7 +1578,7 @@
       <c r="A64" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B64" s="29"/>
+      <c r="B64" s="33"/>
       <c r="C64" s="22">
         <f>SUM(C59:C63)</f>
         <v>0</v>
@@ -1568,42 +1590,42 @@
       <c r="A65" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B65" s="30"/>
+      <c r="B65" s="34"/>
       <c r="C65" s="25"/>
       <c r="D65" s="26"/>
       <c r="E65" s="27"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="4"/>
-      <c r="B66" s="28"/>
+      <c r="B66" s="32"/>
       <c r="C66" s="5"/>
       <c r="D66" s="6"/>
       <c r="E66" s="21"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="7"/>
-      <c r="B67" s="29"/>
+      <c r="B67" s="33"/>
       <c r="C67" s="8"/>
       <c r="D67" s="9"/>
       <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" s="7"/>
-      <c r="B68" s="29"/>
+      <c r="B68" s="33"/>
       <c r="C68" s="8"/>
       <c r="D68" s="9"/>
       <c r="E68" s="8"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="7"/>
-      <c r="B69" s="29"/>
+      <c r="B69" s="33"/>
       <c r="C69" s="8"/>
       <c r="D69" s="9"/>
       <c r="E69" s="8"/>
     </row>
     <row r="70" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="10"/>
-      <c r="B70" s="29"/>
+      <c r="B70" s="33"/>
       <c r="C70" s="10"/>
       <c r="D70" s="11"/>
       <c r="E70" s="10"/>
@@ -1612,7 +1634,7 @@
       <c r="A71" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B71" s="29"/>
+      <c r="B71" s="33"/>
       <c r="C71" s="22">
         <f>SUM(C66:C70)</f>
         <v>0</v>
@@ -1624,19 +1646,19 @@
       <c r="A72" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B72" s="30"/>
+      <c r="B72" s="34"/>
       <c r="C72" s="25"/>
       <c r="D72" s="26"/>
       <c r="E72" s="27"/>
     </row>
     <row r="73" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="31" t="s">
+      <c r="A73" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="B73" s="32"/>
+      <c r="B73" s="36"/>
       <c r="C73" s="13">
         <f>MROUND(SUM(C6:C72) /8,0.2)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D73" s="14"/>
       <c r="E73" s="15"/>
@@ -1651,6 +1673,31 @@
     </row>
   </sheetData>
   <mergeCells count="41">
+    <mergeCell ref="D64:E64"/>
+    <mergeCell ref="C65:E65"/>
+    <mergeCell ref="B66:B72"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="C72:E72"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="C51:E51"/>
+    <mergeCell ref="B52:B58"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B37"/>
+    <mergeCell ref="B38:B44"/>
+    <mergeCell ref="B45:B51"/>
+    <mergeCell ref="B59:B65"/>
     <mergeCell ref="D43:E43"/>
     <mergeCell ref="C44:E44"/>
     <mergeCell ref="B1:C1"/>
@@ -1667,31 +1714,6 @@
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="C19:E19"/>
-    <mergeCell ref="A73:B73"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B37"/>
-    <mergeCell ref="B38:B44"/>
-    <mergeCell ref="B45:B51"/>
-    <mergeCell ref="B59:B65"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="B52:B58"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="C58:E58"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="B66:B72"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="C72:E72"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C66:C71 B13 B16 B20 B24 B28 B31 C31:C36 B38 C38:C43 B45 C45:C50 B52 C52:C57 B59 C59:C64 B66 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1710,6 +1732,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -1871,12 +1899,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1887,6 +1909,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1904,15 +1935,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat(avancée v2): avancée de la v2 modulaire avec la création de différentes classes
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B047783D-5BBA-4ADC-BFED-A86340BF2EDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3000251-9CA5-45B5-B075-BCA2383FC490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5985" yWindow="1710" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$73</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$70</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="52">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -200,6 +200,12 @@
   </si>
   <si>
     <t>Avancée de nouvelles choses et corrections de nouveaux bugs rencontrés</t>
+  </si>
+  <si>
+    <t>Transformation du fichier d'un code en vrac à un code contenant des classes</t>
+  </si>
+  <si>
+    <t>Rendu de la v1</t>
   </si>
 </sst>
 </file>
@@ -890,7 +896,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" style="1" customWidth="1"/>
@@ -1301,7 +1307,9 @@
       <c r="A31" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="32"/>
+      <c r="B31" s="32">
+        <v>46050</v>
+      </c>
       <c r="C31" s="5">
         <v>6</v>
       </c>
@@ -1312,7 +1320,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>31</v>
       </c>
@@ -1327,384 +1335,373 @@
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="7"/>
+    <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="12" t="s">
+        <v>22</v>
+      </c>
       <c r="B33" s="33"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="9"/>
-      <c r="E33" s="8"/>
-    </row>
-    <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="7"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="9"/>
-      <c r="E34" s="8"/>
-    </row>
-    <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="10"/>
-      <c r="B35" s="33"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="10"/>
-    </row>
-    <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
+      <c r="C33" s="22">
+        <f>SUM(C31:C32)</f>
+        <v>12</v>
+      </c>
+      <c r="D33" s="23"/>
+      <c r="E33" s="24"/>
+    </row>
+    <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B34" s="34"/>
+      <c r="C34" s="25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D34" s="26"/>
+      <c r="E34" s="27"/>
+    </row>
+    <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" s="32">
+        <v>46057</v>
+      </c>
+      <c r="C35" s="5">
+        <v>6</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E35" s="21"/>
+    </row>
+    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="7"/>
+      <c r="B36" s="33"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="8"/>
+    </row>
+    <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="7"/>
+      <c r="B37" s="33"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="8"/>
+    </row>
+    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="7"/>
+      <c r="B38" s="33"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="8"/>
+    </row>
+    <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="10"/>
+      <c r="B39" s="33"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="11"/>
+      <c r="E39" s="10"/>
+    </row>
+    <row r="40" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="33"/>
-      <c r="C36" s="22">
-        <f>SUM(C31:C35)</f>
+      <c r="B40" s="33"/>
+      <c r="C40" s="22">
+        <f>SUM(C35:C39)</f>
+        <v>6</v>
+      </c>
+      <c r="D40" s="23"/>
+      <c r="E40" s="24"/>
+    </row>
+    <row r="41" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" s="34"/>
+      <c r="C41" s="25"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="27"/>
+    </row>
+    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="4"/>
+      <c r="B42" s="32"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="21"/>
+    </row>
+    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="7"/>
+      <c r="B43" s="33"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="8"/>
+    </row>
+    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="7"/>
+      <c r="B44" s="33"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="8"/>
+    </row>
+    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="7"/>
+      <c r="B45" s="33"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="8"/>
+    </row>
+    <row r="46" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="10"/>
+      <c r="B46" s="33"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="10"/>
+    </row>
+    <row r="47" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B47" s="33"/>
+      <c r="C47" s="22">
+        <f>SUM(C42:C46)</f>
+        <v>0</v>
+      </c>
+      <c r="D47" s="23"/>
+      <c r="E47" s="24"/>
+    </row>
+    <row r="48" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48" s="34"/>
+      <c r="C48" s="25"/>
+      <c r="D48" s="26"/>
+      <c r="E48" s="27"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="4"/>
+      <c r="B49" s="32"/>
+      <c r="C49" s="5"/>
+      <c r="D49" s="6"/>
+      <c r="E49" s="21"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="7"/>
+      <c r="B50" s="33"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="8"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="7"/>
+      <c r="B51" s="33"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="8"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="7"/>
+      <c r="B52" s="33"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="8"/>
+    </row>
+    <row r="53" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="10"/>
+      <c r="B53" s="33"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="11"/>
+      <c r="E53" s="10"/>
+    </row>
+    <row r="54" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B54" s="33"/>
+      <c r="C54" s="22">
+        <f>SUM(C49:C53)</f>
+        <v>0</v>
+      </c>
+      <c r="D54" s="23"/>
+      <c r="E54" s="24"/>
+    </row>
+    <row r="55" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B55" s="34"/>
+      <c r="C55" s="25"/>
+      <c r="D55" s="26"/>
+      <c r="E55" s="27"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D36" s="23"/>
-      <c r="E36" s="24"/>
-    </row>
-    <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
+      <c r="B56" s="32"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="6"/>
+      <c r="E56" s="21"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="7"/>
+      <c r="B57" s="33"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="8"/>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="7"/>
+      <c r="B58" s="33"/>
+      <c r="C58" s="8"/>
+      <c r="D58" s="9"/>
+      <c r="E58" s="8"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="7"/>
+      <c r="B59" s="33"/>
+      <c r="C59" s="8"/>
+      <c r="D59" s="9"/>
+      <c r="E59" s="8"/>
+    </row>
+    <row r="60" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="10"/>
+      <c r="B60" s="33"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="10"/>
+    </row>
+    <row r="61" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B61" s="33"/>
+      <c r="C61" s="22">
+        <f>SUM(C56:C60)</f>
+        <v>0</v>
+      </c>
+      <c r="D61" s="23"/>
+      <c r="E61" s="24"/>
+    </row>
+    <row r="62" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B37" s="34"/>
-      <c r="C37" s="25"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="27"/>
-    </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="4"/>
-      <c r="B38" s="32"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="6"/>
-      <c r="E38" s="21"/>
-    </row>
-    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="7"/>
-      <c r="B39" s="33"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="8"/>
-    </row>
-    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="7"/>
-      <c r="B40" s="33"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="8"/>
-    </row>
-    <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="7"/>
-      <c r="B41" s="33"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="8"/>
-    </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="10"/>
-      <c r="B42" s="33"/>
-      <c r="C42" s="10"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="10"/>
-    </row>
-    <row r="43" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="12" t="s">
+      <c r="B62" s="34"/>
+      <c r="C62" s="25"/>
+      <c r="D62" s="26"/>
+      <c r="E62" s="27"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="4"/>
+      <c r="B63" s="32"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="6"/>
+      <c r="E63" s="21"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="7"/>
+      <c r="B64" s="33"/>
+      <c r="C64" s="8"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="8"/>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="7"/>
+      <c r="B65" s="33"/>
+      <c r="C65" s="8"/>
+      <c r="D65" s="9"/>
+      <c r="E65" s="8"/>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="7"/>
+      <c r="B66" s="33"/>
+      <c r="C66" s="8"/>
+      <c r="D66" s="9"/>
+      <c r="E66" s="8"/>
+    </row>
+    <row r="67" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="10"/>
+      <c r="B67" s="33"/>
+      <c r="C67" s="10"/>
+      <c r="D67" s="11"/>
+      <c r="E67" s="10"/>
+    </row>
+    <row r="68" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B43" s="33"/>
-      <c r="C43" s="22">
-        <f>SUM(C38:C42)</f>
+      <c r="B68" s="33"/>
+      <c r="C68" s="22">
+        <f>SUM(C63:C67)</f>
         <v>0</v>
       </c>
-      <c r="D43" s="23"/>
-      <c r="E43" s="24"/>
-    </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="12" t="s">
+      <c r="D68" s="23"/>
+      <c r="E68" s="24"/>
+    </row>
+    <row r="69" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B44" s="34"/>
-      <c r="C44" s="25"/>
-      <c r="D44" s="26"/>
-      <c r="E44" s="27"/>
-    </row>
-    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="4"/>
-      <c r="B45" s="32"/>
-      <c r="C45" s="5"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="21"/>
-    </row>
-    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="7"/>
-      <c r="B46" s="33"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="8"/>
-    </row>
-    <row r="47" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="7"/>
-      <c r="B47" s="33"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="9"/>
-      <c r="E47" s="8"/>
-    </row>
-    <row r="48" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="7"/>
-      <c r="B48" s="33"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="9"/>
-      <c r="E48" s="8"/>
-    </row>
-    <row r="49" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="10"/>
-      <c r="B49" s="33"/>
-      <c r="C49" s="10"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="10"/>
-    </row>
-    <row r="50" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B50" s="33"/>
-      <c r="C50" s="22">
-        <f>SUM(C45:C49)</f>
-        <v>0</v>
-      </c>
-      <c r="D50" s="23"/>
-      <c r="E50" s="24"/>
-    </row>
-    <row r="51" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B51" s="34"/>
-      <c r="C51" s="25"/>
-      <c r="D51" s="26"/>
-      <c r="E51" s="27"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="4"/>
-      <c r="B52" s="32"/>
-      <c r="C52" s="5"/>
-      <c r="D52" s="6"/>
-      <c r="E52" s="21"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="7"/>
-      <c r="B53" s="33"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="8"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="7"/>
-      <c r="B54" s="33"/>
-      <c r="C54" s="8"/>
-      <c r="D54" s="9"/>
-      <c r="E54" s="8"/>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="7"/>
-      <c r="B55" s="33"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="9"/>
-      <c r="E55" s="8"/>
-    </row>
-    <row r="56" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="10"/>
-      <c r="B56" s="33"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="10"/>
-    </row>
-    <row r="57" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B57" s="33"/>
-      <c r="C57" s="22">
-        <f>SUM(C52:C56)</f>
-        <v>0</v>
-      </c>
-      <c r="D57" s="23"/>
-      <c r="E57" s="24"/>
-    </row>
-    <row r="58" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B58" s="34"/>
-      <c r="C58" s="25"/>
-      <c r="D58" s="26"/>
-      <c r="E58" s="27"/>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B59" s="32"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="21"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="7"/>
-      <c r="B60" s="33"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="8"/>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="7"/>
-      <c r="B61" s="33"/>
-      <c r="C61" s="8"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="8"/>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="7"/>
-      <c r="B62" s="33"/>
-      <c r="C62" s="8"/>
-      <c r="D62" s="9"/>
-      <c r="E62" s="8"/>
-    </row>
-    <row r="63" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="10"/>
-      <c r="B63" s="33"/>
-      <c r="C63" s="10"/>
-      <c r="D63" s="11"/>
-      <c r="E63" s="10"/>
-    </row>
-    <row r="64" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B64" s="33"/>
-      <c r="C64" s="22">
-        <f>SUM(C59:C63)</f>
-        <v>0</v>
-      </c>
-      <c r="D64" s="23"/>
-      <c r="E64" s="24"/>
-    </row>
-    <row r="65" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B65" s="34"/>
-      <c r="C65" s="25"/>
-      <c r="D65" s="26"/>
-      <c r="E65" s="27"/>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="4"/>
-      <c r="B66" s="32"/>
-      <c r="C66" s="5"/>
-      <c r="D66" s="6"/>
-      <c r="E66" s="21"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="7"/>
-      <c r="B67" s="33"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="8"/>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="7"/>
-      <c r="B68" s="33"/>
-      <c r="C68" s="8"/>
-      <c r="D68" s="9"/>
-      <c r="E68" s="8"/>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="7"/>
-      <c r="B69" s="33"/>
-      <c r="C69" s="8"/>
-      <c r="D69" s="9"/>
-      <c r="E69" s="8"/>
-    </row>
-    <row r="70" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="10"/>
-      <c r="B70" s="33"/>
-      <c r="C70" s="10"/>
-      <c r="D70" s="11"/>
-      <c r="E70" s="10"/>
-    </row>
-    <row r="71" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B71" s="33"/>
-      <c r="C71" s="22">
-        <f>SUM(C66:C70)</f>
-        <v>0</v>
-      </c>
-      <c r="D71" s="23"/>
-      <c r="E71" s="24"/>
-    </row>
-    <row r="72" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B72" s="34"/>
-      <c r="C72" s="25"/>
-      <c r="D72" s="26"/>
-      <c r="E72" s="27"/>
-    </row>
-    <row r="73" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="35" t="s">
+      <c r="B69" s="34"/>
+      <c r="C69" s="25"/>
+      <c r="D69" s="26"/>
+      <c r="E69" s="27"/>
+    </row>
+    <row r="70" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="35" t="s">
         <v>14</v>
       </c>
-      <c r="B73" s="36"/>
-      <c r="C73" s="13">
-        <f>MROUND(SUM(C6:C72) /8,0.2)</f>
-        <v>12</v>
-      </c>
-      <c r="D73" s="14"/>
-      <c r="E73" s="15"/>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="16" t="s">
+      <c r="B70" s="36"/>
+      <c r="C70" s="13">
+        <f>MROUND(SUM(C6:C69) /8,0.2)</f>
+        <v>13.600000000000001</v>
+      </c>
+      <c r="D70" s="14"/>
+      <c r="E70" s="15"/>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="16" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="16"/>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="C65:E65"/>
-    <mergeCell ref="B66:B72"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="C72:E72"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="C51:E51"/>
-    <mergeCell ref="B52:B58"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="B63:B69"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="B49:B55"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="C55:E55"/>
     <mergeCell ref="B20:B23"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="C23:E23"/>
-    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D33:E33"/>
     <mergeCell ref="D26:E26"/>
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="C30:E30"/>
-    <mergeCell ref="A73:B73"/>
+    <mergeCell ref="A70:B70"/>
     <mergeCell ref="B24:B27"/>
     <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B37"/>
-    <mergeCell ref="B38:B44"/>
-    <mergeCell ref="B45:B51"/>
-    <mergeCell ref="B59:B65"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="C44:E44"/>
+    <mergeCell ref="B31:B34"/>
+    <mergeCell ref="B35:B41"/>
+    <mergeCell ref="B42:B48"/>
+    <mergeCell ref="B56:B62"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="C41:E41"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C34:E34"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="B6:B12"/>
@@ -1716,7 +1713,7 @@
     <mergeCell ref="C19:E19"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C66:C71 B13 B16 B20 B24 B28 B31 C31:C36 B38 C38:C43 B45 C45:C50 B52 C52:C57 B59 C59:C64 B66 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C63:C68 B13 B16 B20 B24 B28 B31 B35 C35:C40 B42 C42:C47 B49 C49:C54 B56 C56:C61 B63 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C33" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(classes & ajouts): modification des dernières fonctions en classes, modifications de certaines de celle-ci avec quelques ajustements et ajout de nouvelles classes
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3000251-9CA5-45B5-B075-BCA2383FC490}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC7DF255-8836-4F24-8C76-60F86E853C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="53">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t>Rendu de la v1</t>
+  </si>
+  <si>
+    <t>Mise en place de nouvelle classe et amélioration du code dans certaines fonctionnalités</t>
   </si>
 </sst>
 </file>
@@ -550,18 +553,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -579,6 +570,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -913,10 +916,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="28"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -926,10 +929,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -941,10 +944,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="28"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -956,12 +959,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -984,7 +987,7 @@
       <c r="A6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="28">
         <v>45671</v>
       </c>
       <c r="C6" s="5">
@@ -999,7 +1002,7 @@
       <c r="A7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -1012,7 +1015,7 @@
       <c r="A8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="33"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="8">
         <v>3</v>
       </c>
@@ -1025,7 +1028,7 @@
       <c r="A9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="33"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="8">
         <v>1</v>
       </c>
@@ -1038,7 +1041,7 @@
       <c r="A10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="33"/>
+      <c r="B10" s="29"/>
       <c r="C10" s="10">
         <v>2</v>
       </c>
@@ -1053,7 +1056,7 @@
       <c r="A11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1065,7 +1068,7 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="34"/>
+      <c r="B12" s="30"/>
       <c r="C12" s="25" t="s">
         <v>33</v>
       </c>
@@ -1076,7 +1079,7 @@
       <c r="A13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="28">
         <v>45678</v>
       </c>
       <c r="C13" s="5">
@@ -1093,7 +1096,7 @@
       <c r="A14" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="33"/>
+      <c r="B14" s="29"/>
       <c r="C14" s="22">
         <f>SUM(C13:C13)</f>
         <v>6</v>
@@ -1105,7 +1108,7 @@
       <c r="A15" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="34"/>
+      <c r="B15" s="30"/>
       <c r="C15" s="25" t="s">
         <v>34</v>
       </c>
@@ -1116,7 +1119,7 @@
       <c r="A16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="32">
+      <c r="B16" s="28">
         <v>45681</v>
       </c>
       <c r="C16" s="5">
@@ -1131,7 +1134,7 @@
       <c r="A17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="33"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="8">
         <v>2</v>
       </c>
@@ -1144,7 +1147,7 @@
       <c r="A18" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="33"/>
+      <c r="B18" s="29"/>
       <c r="C18" s="22">
         <f>SUM(C16:C17)</f>
         <v>6</v>
@@ -1156,7 +1159,7 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="34"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="25" t="s">
         <v>38</v>
       </c>
@@ -1167,7 +1170,7 @@
       <c r="A20" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="28">
         <v>45682</v>
       </c>
       <c r="C20" s="5">
@@ -1182,7 +1185,7 @@
       <c r="A21" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="33"/>
+      <c r="B21" s="29"/>
       <c r="C21" s="8">
         <v>2</v>
       </c>
@@ -1195,7 +1198,7 @@
       <c r="A22" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="33"/>
+      <c r="B22" s="29"/>
       <c r="C22" s="22">
         <f>SUM(C20:C21)</f>
         <v>6</v>
@@ -1207,7 +1210,7 @@
       <c r="A23" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="34"/>
+      <c r="B23" s="30"/>
       <c r="C23" s="25" t="s">
         <v>39</v>
       </c>
@@ -1218,7 +1221,7 @@
       <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="32">
+      <c r="B24" s="28">
         <v>46048</v>
       </c>
       <c r="C24" s="5">
@@ -1233,7 +1236,7 @@
       <c r="A25" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="33"/>
+      <c r="B25" s="29"/>
       <c r="C25" s="8">
         <v>2</v>
       </c>
@@ -1246,7 +1249,7 @@
       <c r="A26" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="33"/>
+      <c r="B26" s="29"/>
       <c r="C26" s="22">
         <f>SUM(C24:C25)</f>
         <v>4</v>
@@ -1258,7 +1261,7 @@
       <c r="A27" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B27" s="34"/>
+      <c r="B27" s="30"/>
       <c r="C27" s="25" t="s">
         <v>45</v>
       </c>
@@ -1269,7 +1272,7 @@
       <c r="A28" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="32">
+      <c r="B28" s="28">
         <v>46049</v>
       </c>
       <c r="C28" s="5">
@@ -1284,7 +1287,7 @@
       <c r="A29" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="33"/>
+      <c r="B29" s="29"/>
       <c r="C29" s="22">
         <f>SUM(C28:C28)</f>
         <v>2</v>
@@ -1296,7 +1299,7 @@
       <c r="A30" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="34"/>
+      <c r="B30" s="30"/>
       <c r="C30" s="25" t="s">
         <v>46</v>
       </c>
@@ -1307,7 +1310,7 @@
       <c r="A31" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="32">
+      <c r="B31" s="28">
         <v>46050</v>
       </c>
       <c r="C31" s="5">
@@ -1324,7 +1327,7 @@
       <c r="A32" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="33"/>
+      <c r="B32" s="29"/>
       <c r="C32" s="8">
         <v>6</v>
       </c>
@@ -1339,7 +1342,7 @@
       <c r="A33" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B33" s="33"/>
+      <c r="B33" s="29"/>
       <c r="C33" s="22">
         <f>SUM(C31:C32)</f>
         <v>12</v>
@@ -1351,7 +1354,7 @@
       <c r="A34" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="34"/>
+      <c r="B34" s="30"/>
       <c r="C34" s="25" t="s">
         <v>51</v>
       </c>
@@ -1362,7 +1365,7 @@
       <c r="A35" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="32">
+      <c r="B35" s="28">
         <v>46057</v>
       </c>
       <c r="C35" s="5">
@@ -1371,32 +1374,34 @@
       <c r="D35" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E35" s="21"/>
+      <c r="E35" s="10" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="33"/>
+      <c r="B36" s="29"/>
       <c r="C36" s="8"/>
       <c r="D36" s="9"/>
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="33"/>
+      <c r="B37" s="29"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7"/>
-      <c r="B38" s="33"/>
+      <c r="B38" s="29"/>
       <c r="C38" s="8"/>
       <c r="D38" s="9"/>
       <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="10"/>
-      <c r="B39" s="33"/>
+      <c r="B39" s="29"/>
       <c r="C39" s="10"/>
       <c r="D39" s="11"/>
       <c r="E39" s="10"/>
@@ -1405,7 +1410,7 @@
       <c r="A40" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B40" s="33"/>
+      <c r="B40" s="29"/>
       <c r="C40" s="22">
         <f>SUM(C35:C39)</f>
         <v>6</v>
@@ -1417,42 +1422,52 @@
       <c r="A41" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="34"/>
+      <c r="B41" s="30"/>
       <c r="C41" s="25"/>
       <c r="D41" s="26"/>
       <c r="E41" s="27"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="4"/>
-      <c r="B42" s="32"/>
-      <c r="C42" s="5"/>
-      <c r="D42" s="6"/>
-      <c r="E42" s="21"/>
+      <c r="A42" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B42" s="28">
+        <v>46062</v>
+      </c>
+      <c r="C42" s="5">
+        <v>9</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E42" s="10" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
-      <c r="B43" s="33"/>
+      <c r="B43" s="29"/>
       <c r="C43" s="8"/>
       <c r="D43" s="9"/>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
-      <c r="B44" s="33"/>
+      <c r="B44" s="29"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7"/>
-      <c r="B45" s="33"/>
+      <c r="B45" s="29"/>
       <c r="C45" s="8"/>
       <c r="D45" s="9"/>
       <c r="E45" s="8"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="10"/>
-      <c r="B46" s="33"/>
+      <c r="B46" s="29"/>
       <c r="C46" s="10"/>
       <c r="D46" s="11"/>
       <c r="E46" s="10"/>
@@ -1461,10 +1476,10 @@
       <c r="A47" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B47" s="33"/>
+      <c r="B47" s="29"/>
       <c r="C47" s="22">
         <f>SUM(C42:C46)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D47" s="23"/>
       <c r="E47" s="24"/>
@@ -1473,42 +1488,42 @@
       <c r="A48" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B48" s="34"/>
+      <c r="B48" s="30"/>
       <c r="C48" s="25"/>
       <c r="D48" s="26"/>
       <c r="E48" s="27"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
-      <c r="B49" s="32"/>
+      <c r="B49" s="28"/>
       <c r="C49" s="5"/>
       <c r="D49" s="6"/>
       <c r="E49" s="21"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="33"/>
+      <c r="B50" s="29"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="33"/>
+      <c r="B51" s="29"/>
       <c r="C51" s="8"/>
       <c r="D51" s="9"/>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="7"/>
-      <c r="B52" s="33"/>
+      <c r="B52" s="29"/>
       <c r="C52" s="8"/>
       <c r="D52" s="9"/>
       <c r="E52" s="8"/>
     </row>
     <row r="53" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="10"/>
-      <c r="B53" s="33"/>
+      <c r="B53" s="29"/>
       <c r="C53" s="10"/>
       <c r="D53" s="11"/>
       <c r="E53" s="10"/>
@@ -1517,7 +1532,7 @@
       <c r="A54" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B54" s="33"/>
+      <c r="B54" s="29"/>
       <c r="C54" s="22">
         <f>SUM(C49:C53)</f>
         <v>0</v>
@@ -1529,7 +1544,7 @@
       <c r="A55" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B55" s="34"/>
+      <c r="B55" s="30"/>
       <c r="C55" s="25"/>
       <c r="D55" s="26"/>
       <c r="E55" s="27"/>
@@ -1538,35 +1553,35 @@
       <c r="A56" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B56" s="32"/>
+      <c r="B56" s="28"/>
       <c r="C56" s="5"/>
       <c r="D56" s="6"/>
       <c r="E56" s="21"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="33"/>
+      <c r="B57" s="29"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="33"/>
+      <c r="B58" s="29"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="7"/>
-      <c r="B59" s="33"/>
+      <c r="B59" s="29"/>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
       <c r="E59" s="8"/>
     </row>
     <row r="60" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="10"/>
-      <c r="B60" s="33"/>
+      <c r="B60" s="29"/>
       <c r="C60" s="10"/>
       <c r="D60" s="11"/>
       <c r="E60" s="10"/>
@@ -1575,7 +1590,7 @@
       <c r="A61" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B61" s="33"/>
+      <c r="B61" s="29"/>
       <c r="C61" s="22">
         <f>SUM(C56:C60)</f>
         <v>0</v>
@@ -1587,42 +1602,42 @@
       <c r="A62" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B62" s="34"/>
+      <c r="B62" s="30"/>
       <c r="C62" s="25"/>
       <c r="D62" s="26"/>
       <c r="E62" s="27"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="4"/>
-      <c r="B63" s="32"/>
+      <c r="B63" s="28"/>
       <c r="C63" s="5"/>
       <c r="D63" s="6"/>
       <c r="E63" s="21"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="33"/>
+      <c r="B64" s="29"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="33"/>
+      <c r="B65" s="29"/>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
-      <c r="B66" s="33"/>
+      <c r="B66" s="29"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
     <row r="67" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="10"/>
-      <c r="B67" s="33"/>
+      <c r="B67" s="29"/>
       <c r="C67" s="10"/>
       <c r="D67" s="11"/>
       <c r="E67" s="10"/>
@@ -1631,7 +1646,7 @@
       <c r="A68" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B68" s="33"/>
+      <c r="B68" s="29"/>
       <c r="C68" s="22">
         <f>SUM(C63:C67)</f>
         <v>0</v>
@@ -1643,19 +1658,19 @@
       <c r="A69" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B69" s="34"/>
+      <c r="B69" s="30"/>
       <c r="C69" s="25"/>
       <c r="D69" s="26"/>
       <c r="E69" s="27"/>
     </row>
     <row r="70" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="35" t="s">
+      <c r="A70" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B70" s="36"/>
+      <c r="B70" s="32"/>
       <c r="C70" s="13">
         <f>MROUND(SUM(C6:C69) /8,0.2)</f>
-        <v>13.600000000000001</v>
+        <v>15.8</v>
       </c>
       <c r="D70" s="14"/>
       <c r="E70" s="15"/>
@@ -1670,31 +1685,6 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="B63:B69"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="B49:B55"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="A70:B70"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B34"/>
-    <mergeCell ref="B35:B41"/>
-    <mergeCell ref="B42:B48"/>
-    <mergeCell ref="B56:B62"/>
     <mergeCell ref="D40:E40"/>
     <mergeCell ref="C41:E41"/>
     <mergeCell ref="B1:C1"/>
@@ -1711,6 +1701,31 @@
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="C19:E19"/>
+    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B34"/>
+    <mergeCell ref="B35:B41"/>
+    <mergeCell ref="B42:B48"/>
+    <mergeCell ref="B56:B62"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="B49:B55"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="C62:E62"/>
+    <mergeCell ref="B63:B69"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="C69:E69"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C63:C68 B13 B16 B20 B24 B28 B31 B35 C35:C40 B42 C42:C47 B49 C49:C54 B56 C56:C61 B63 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C33" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1729,12 +1744,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -1896,6 +1905,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1906,15 +1921,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1932,6 +1938,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat(v2 terminée): Dernière finition nécessaire à la v2 + implémentation du projectile
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC7DF255-8836-4F24-8C76-60F86E853C77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D3FA3D-D46F-41E6-8E5F-2DF762D19B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34635" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$70</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$71</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="60">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -196,9 +196,6 @@
     <t xml:space="preserve">Commit réalisé </t>
   </si>
   <si>
-    <t>Validation des dernières modifs pour la v1 + rendu v1</t>
-  </si>
-  <si>
     <t>Avancée de nouvelles choses et corrections de nouveaux bugs rencontrés</t>
   </si>
   <si>
@@ -209,6 +206,30 @@
   </si>
   <si>
     <t>Mise en place de nouvelle classe et amélioration du code dans certaines fonctionnalités</t>
+  </si>
+  <si>
+    <t>Implémentation du projectile de la tour</t>
+  </si>
+  <si>
+    <t>Rendu v2</t>
+  </si>
+  <si>
+    <t>Rendu v1</t>
+  </si>
+  <si>
+    <t>Validation des dernières modifs pour la v1</t>
+  </si>
+  <si>
+    <t>Realease v1 GitHub</t>
+  </si>
+  <si>
+    <t>Realease v2 GitHub</t>
+  </si>
+  <si>
+    <t>Word</t>
+  </si>
+  <si>
+    <t>Amélioration de l'intro + Mise en page</t>
   </si>
 </sst>
 </file>
@@ -280,7 +301,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -445,6 +466,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="dashed">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -454,7 +488,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -531,6 +565,14 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -899,7 +941,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" style="1" customWidth="1"/>
@@ -916,10 +958,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="33"/>
+      <c r="C1" s="35"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -929,10 +971,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="B2" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="33"/>
+      <c r="C2" s="35"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -944,10 +986,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="33" t="s">
+      <c r="B3" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="35"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -959,12 +1001,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="38"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -987,7 +1029,7 @@
       <c r="A6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="28">
+      <c r="B6" s="30">
         <v>45671</v>
       </c>
       <c r="C6" s="5">
@@ -1002,7 +1044,7 @@
       <c r="A7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="29"/>
+      <c r="B7" s="31"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -1015,7 +1057,7 @@
       <c r="A8" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="29"/>
+      <c r="B8" s="31"/>
       <c r="C8" s="8">
         <v>3</v>
       </c>
@@ -1028,7 +1070,7 @@
       <c r="A9" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="29"/>
+      <c r="B9" s="31"/>
       <c r="C9" s="8">
         <v>1</v>
       </c>
@@ -1041,7 +1083,7 @@
       <c r="A10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="29"/>
+      <c r="B10" s="31"/>
       <c r="C10" s="10">
         <v>2</v>
       </c>
@@ -1056,30 +1098,30 @@
       <c r="A11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="29"/>
+      <c r="B11" s="31"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
       </c>
-      <c r="D11" s="23"/>
-      <c r="E11" s="24"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="26"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="30"/>
-      <c r="C12" s="25" t="s">
+      <c r="B12" s="32"/>
+      <c r="C12" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="26"/>
-      <c r="E12" s="27"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="29"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="30">
         <v>45678</v>
       </c>
       <c r="C13" s="5">
@@ -1096,30 +1138,30 @@
       <c r="A14" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="29"/>
+      <c r="B14" s="31"/>
       <c r="C14" s="22">
         <f>SUM(C13:C13)</f>
         <v>6</v>
       </c>
-      <c r="D14" s="23"/>
-      <c r="E14" s="24"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="26"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="30"/>
-      <c r="C15" s="25" t="s">
+      <c r="B15" s="32"/>
+      <c r="C15" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="26"/>
-      <c r="E15" s="27"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="29"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="28">
+      <c r="B16" s="30">
         <v>45681</v>
       </c>
       <c r="C16" s="5">
@@ -1134,7 +1176,7 @@
       <c r="A17" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="29"/>
+      <c r="B17" s="31"/>
       <c r="C17" s="8">
         <v>2</v>
       </c>
@@ -1147,30 +1189,30 @@
       <c r="A18" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="29"/>
+      <c r="B18" s="31"/>
       <c r="C18" s="22">
         <f>SUM(C16:C17)</f>
         <v>6</v>
       </c>
-      <c r="D18" s="23"/>
-      <c r="E18" s="24"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="26"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="25" t="s">
+      <c r="B19" s="32"/>
+      <c r="C19" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="D19" s="26"/>
-      <c r="E19" s="27"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="29"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="28">
+      <c r="B20" s="30">
         <v>45682</v>
       </c>
       <c r="C20" s="5">
@@ -1185,7 +1227,7 @@
       <c r="A21" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="29"/>
+      <c r="B21" s="31"/>
       <c r="C21" s="8">
         <v>2</v>
       </c>
@@ -1198,30 +1240,30 @@
       <c r="A22" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="29"/>
+      <c r="B22" s="31"/>
       <c r="C22" s="22">
         <f>SUM(C20:C21)</f>
         <v>6</v>
       </c>
-      <c r="D22" s="23"/>
-      <c r="E22" s="24"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="26"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="30"/>
-      <c r="C23" s="25" t="s">
+      <c r="B23" s="32"/>
+      <c r="C23" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="D23" s="26"/>
-      <c r="E23" s="27"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="29"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B24" s="28">
+      <c r="B24" s="30">
         <v>46048</v>
       </c>
       <c r="C24" s="5">
@@ -1236,7 +1278,7 @@
       <c r="A25" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B25" s="29"/>
+      <c r="B25" s="31"/>
       <c r="C25" s="8">
         <v>2</v>
       </c>
@@ -1249,30 +1291,30 @@
       <c r="A26" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="29"/>
+      <c r="B26" s="31"/>
       <c r="C26" s="22">
         <f>SUM(C24:C25)</f>
         <v>4</v>
       </c>
-      <c r="D26" s="23"/>
-      <c r="E26" s="24"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="26"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B27" s="30"/>
-      <c r="C27" s="25" t="s">
+      <c r="B27" s="32"/>
+      <c r="C27" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="D27" s="26"/>
-      <c r="E27" s="27"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="29"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="28">
+      <c r="B28" s="30">
         <v>46049</v>
       </c>
       <c r="C28" s="5">
@@ -1287,411 +1329,448 @@
       <c r="A29" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="29"/>
+      <c r="B29" s="31"/>
       <c r="C29" s="22">
         <f>SUM(C28:C28)</f>
         <v>2</v>
       </c>
-      <c r="D29" s="23"/>
-      <c r="E29" s="24"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="26"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="30"/>
-      <c r="C30" s="25" t="s">
+      <c r="B30" s="32"/>
+      <c r="C30" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="D30" s="26"/>
-      <c r="E30" s="27"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="29"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="28">
+      <c r="B31" s="30">
         <v>46050</v>
       </c>
       <c r="C31" s="5">
         <v>6</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" s="31"/>
+      <c r="C32" s="23">
+        <v>1</v>
+      </c>
+      <c r="D32" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="29"/>
-      <c r="C32" s="8">
-        <v>6</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E32" s="10" t="s">
+      <c r="B33" s="31"/>
+      <c r="C33" s="8">
+        <v>5</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E33" s="10" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B33" s="29"/>
-      <c r="C33" s="22">
-        <f>SUM(C31:C32)</f>
-        <v>12</v>
-      </c>
-      <c r="D33" s="23"/>
-      <c r="E33" s="24"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B34" s="31"/>
+      <c r="C34" s="22">
+        <f>SUM(C31:C33)</f>
+        <v>12</v>
+      </c>
+      <c r="D34" s="25"/>
+      <c r="E34" s="26"/>
+    </row>
+    <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B34" s="30"/>
-      <c r="C34" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="D34" s="26"/>
-      <c r="E34" s="27"/>
-    </row>
-    <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
+      <c r="B35" s="32"/>
+      <c r="C35" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="D35" s="28"/>
+      <c r="E35" s="29"/>
+    </row>
+    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B35" s="28">
+      <c r="B36" s="30">
         <v>46057</v>
       </c>
-      <c r="C35" s="5">
+      <c r="C36" s="5">
         <v>6</v>
       </c>
-      <c r="D35" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E35" s="10" t="s">
+      <c r="D36" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E36" s="10" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="7"/>
-      <c r="B36" s="29"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="9"/>
-      <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="29"/>
+      <c r="B37" s="31"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7"/>
-      <c r="B38" s="29"/>
+      <c r="B38" s="31"/>
       <c r="C38" s="8"/>
       <c r="D38" s="9"/>
       <c r="E38" s="8"/>
     </row>
-    <row r="39" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="10"/>
-      <c r="B39" s="29"/>
-      <c r="C39" s="10"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="10"/>
+    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="7"/>
+      <c r="B39" s="31"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B40" s="29"/>
-      <c r="C40" s="22">
-        <f>SUM(C35:C39)</f>
-        <v>6</v>
-      </c>
-      <c r="D40" s="23"/>
-      <c r="E40" s="24"/>
+      <c r="A40" s="10"/>
+      <c r="B40" s="31"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="11"/>
+      <c r="E40" s="10"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B41" s="31"/>
+      <c r="C41" s="22">
+        <f>SUM(C36:C40)</f>
+        <v>6</v>
+      </c>
+      <c r="D41" s="25"/>
+      <c r="E41" s="26"/>
+    </row>
+    <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B41" s="30"/>
-      <c r="C41" s="25"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="27"/>
-    </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="4" t="s">
+      <c r="B42" s="32"/>
+      <c r="C42" s="27"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="29"/>
+    </row>
+    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B42" s="28">
+      <c r="B43" s="30">
         <v>46062</v>
       </c>
-      <c r="C42" s="5">
+      <c r="C43" s="5">
         <v>9</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="D43" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B44" s="31"/>
+      <c r="C44" s="8">
+        <v>1</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E44" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B45" s="31"/>
+      <c r="C45" s="8">
+        <v>2</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E45" s="8"/>
+    </row>
+    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="7"/>
+      <c r="B46" s="31"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="8"/>
+    </row>
+    <row r="47" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="10"/>
+      <c r="B47" s="31"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="11"/>
+      <c r="E47" s="10"/>
+    </row>
+    <row r="48" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B48" s="31"/>
+      <c r="C48" s="22">
+        <f>SUM(C43:C47)</f>
+        <v>12</v>
+      </c>
+      <c r="D48" s="25"/>
+      <c r="E48" s="26"/>
+    </row>
+    <row r="49" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49" s="32"/>
+      <c r="C49" s="27"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="29"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B50" s="30">
+        <v>46064</v>
+      </c>
+      <c r="C50" s="5">
+        <v>9</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E42" s="10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="7"/>
-      <c r="B43" s="29"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="8"/>
-    </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="7"/>
-      <c r="B44" s="29"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
-      <c r="E44" s="8"/>
-    </row>
-    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="7"/>
-      <c r="B45" s="29"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="8"/>
-    </row>
-    <row r="46" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="10"/>
-      <c r="B46" s="29"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="11"/>
-      <c r="E46" s="10"/>
-    </row>
-    <row r="47" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B47" s="29"/>
-      <c r="C47" s="22">
-        <f>SUM(C42:C46)</f>
-        <v>9</v>
-      </c>
-      <c r="D47" s="23"/>
-      <c r="E47" s="24"/>
-    </row>
-    <row r="48" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B48" s="30"/>
-      <c r="C48" s="25"/>
-      <c r="D48" s="26"/>
-      <c r="E48" s="27"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="4"/>
-      <c r="B49" s="28"/>
-      <c r="C49" s="5"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="21"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="7"/>
-      <c r="B50" s="29"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
-      <c r="E50" s="8"/>
+      <c r="E50" s="21"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="29"/>
+      <c r="B51" s="31"/>
       <c r="C51" s="8"/>
       <c r="D51" s="9"/>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="7"/>
-      <c r="B52" s="29"/>
+      <c r="B52" s="31"/>
       <c r="C52" s="8"/>
       <c r="D52" s="9"/>
       <c r="E52" s="8"/>
     </row>
-    <row r="53" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="10"/>
-      <c r="B53" s="29"/>
-      <c r="C53" s="10"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="10"/>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="7"/>
+      <c r="B53" s="31"/>
+      <c r="C53" s="8"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="8"/>
     </row>
     <row r="54" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B54" s="29"/>
-      <c r="C54" s="22">
-        <f>SUM(C49:C53)</f>
-        <v>0</v>
-      </c>
-      <c r="D54" s="23"/>
-      <c r="E54" s="24"/>
+      <c r="A54" s="10"/>
+      <c r="B54" s="31"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="10"/>
     </row>
     <row r="55" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B55" s="31"/>
+      <c r="C55" s="22">
+        <f>SUM(C50:C54)</f>
+        <v>9</v>
+      </c>
+      <c r="D55" s="25"/>
+      <c r="E55" s="26"/>
+    </row>
+    <row r="56" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B55" s="30"/>
-      <c r="C55" s="25"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="27"/>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
+      <c r="B56" s="32"/>
+      <c r="C56" s="27"/>
+      <c r="D56" s="28"/>
+      <c r="E56" s="29"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B56" s="28"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="6"/>
-      <c r="E56" s="21"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="7"/>
-      <c r="B57" s="29"/>
-      <c r="C57" s="8"/>
-      <c r="D57" s="9"/>
-      <c r="E57" s="8"/>
+      <c r="B57" s="30"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="21"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="29"/>
+      <c r="B58" s="31"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="7"/>
-      <c r="B59" s="29"/>
+      <c r="B59" s="31"/>
       <c r="C59" s="8"/>
       <c r="D59" s="9"/>
       <c r="E59" s="8"/>
     </row>
-    <row r="60" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="10"/>
-      <c r="B60" s="29"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="11"/>
-      <c r="E60" s="10"/>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="7"/>
+      <c r="B60" s="31"/>
+      <c r="C60" s="8"/>
+      <c r="D60" s="9"/>
+      <c r="E60" s="8"/>
     </row>
     <row r="61" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B61" s="29"/>
-      <c r="C61" s="22">
-        <f>SUM(C56:C60)</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="23"/>
-      <c r="E61" s="24"/>
+      <c r="A61" s="10"/>
+      <c r="B61" s="31"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="11"/>
+      <c r="E61" s="10"/>
     </row>
     <row r="62" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B62" s="31"/>
+      <c r="C62" s="22">
+        <f>SUM(C57:C61)</f>
+        <v>0</v>
+      </c>
+      <c r="D62" s="25"/>
+      <c r="E62" s="26"/>
+    </row>
+    <row r="63" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B62" s="30"/>
-      <c r="C62" s="25"/>
-      <c r="D62" s="26"/>
-      <c r="E62" s="27"/>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="4"/>
-      <c r="B63" s="28"/>
-      <c r="C63" s="5"/>
-      <c r="D63" s="6"/>
-      <c r="E63" s="21"/>
+      <c r="B63" s="32"/>
+      <c r="C63" s="27"/>
+      <c r="D63" s="28"/>
+      <c r="E63" s="29"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="7"/>
-      <c r="B64" s="29"/>
-      <c r="C64" s="8"/>
-      <c r="D64" s="9"/>
-      <c r="E64" s="8"/>
+      <c r="A64" s="4"/>
+      <c r="B64" s="30"/>
+      <c r="C64" s="5"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="21"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="29"/>
+      <c r="B65" s="31"/>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
-      <c r="B66" s="29"/>
+      <c r="B66" s="31"/>
       <c r="C66" s="8"/>
       <c r="D66" s="9"/>
       <c r="E66" s="8"/>
     </row>
-    <row r="67" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="10"/>
-      <c r="B67" s="29"/>
-      <c r="C67" s="10"/>
-      <c r="D67" s="11"/>
-      <c r="E67" s="10"/>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="7"/>
+      <c r="B67" s="31"/>
+      <c r="C67" s="8"/>
+      <c r="D67" s="9"/>
+      <c r="E67" s="8"/>
     </row>
     <row r="68" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B68" s="29"/>
-      <c r="C68" s="22">
-        <f>SUM(C63:C67)</f>
-        <v>0</v>
-      </c>
-      <c r="D68" s="23"/>
-      <c r="E68" s="24"/>
+      <c r="A68" s="10"/>
+      <c r="B68" s="31"/>
+      <c r="C68" s="10"/>
+      <c r="D68" s="11"/>
+      <c r="E68" s="10"/>
     </row>
     <row r="69" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B69" s="31"/>
+      <c r="C69" s="22">
+        <f>SUM(C64:C68)</f>
+        <v>0</v>
+      </c>
+      <c r="D69" s="25"/>
+      <c r="E69" s="26"/>
+    </row>
+    <row r="70" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B69" s="30"/>
-      <c r="C69" s="25"/>
-      <c r="D69" s="26"/>
-      <c r="E69" s="27"/>
-    </row>
-    <row r="70" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="31" t="s">
+      <c r="B70" s="32"/>
+      <c r="C70" s="27"/>
+      <c r="D70" s="28"/>
+      <c r="E70" s="29"/>
+    </row>
+    <row r="71" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="B70" s="32"/>
-      <c r="C70" s="13">
-        <f>MROUND(SUM(C6:C69) /8,0.2)</f>
-        <v>15.8</v>
-      </c>
-      <c r="D70" s="14"/>
-      <c r="E70" s="15"/>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="16" t="s">
+      <c r="B71" s="34"/>
+      <c r="C71" s="13">
+        <f>MROUND(SUM(C6:C70) /8,0.2)</f>
+        <v>18.8</v>
+      </c>
+      <c r="D71" s="14"/>
+      <c r="E71" s="15"/>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="16" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="16"/>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="C41:E41"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="C42:E42"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:E4"/>
-    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C35:E35"/>
     <mergeCell ref="D11:E11"/>
     <mergeCell ref="C12:E12"/>
     <mergeCell ref="B6:B12"/>
@@ -1701,34 +1780,34 @@
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="C19:E19"/>
-    <mergeCell ref="A70:B70"/>
+    <mergeCell ref="A71:B71"/>
     <mergeCell ref="B24:B27"/>
     <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B34"/>
-    <mergeCell ref="B35:B41"/>
-    <mergeCell ref="B42:B48"/>
-    <mergeCell ref="B56:B62"/>
+    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="B36:B42"/>
+    <mergeCell ref="B43:B49"/>
+    <mergeCell ref="B57:B63"/>
     <mergeCell ref="B20:B23"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="C23:E23"/>
-    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
     <mergeCell ref="D26:E26"/>
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="C30:E30"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="C48:E48"/>
-    <mergeCell ref="B49:B55"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="C55:E55"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="C62:E62"/>
-    <mergeCell ref="B63:B69"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="C69:E69"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="C49:E49"/>
+    <mergeCell ref="B50:B56"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="C63:E63"/>
+    <mergeCell ref="B64:B70"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="C70:E70"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C63:C68 B13 B16 B20 B24 B28 B31 B35 C35:C40 B42 C42:C47 B49 C49:C54 B56 C56:C61 B63 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C33" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C64:C69 B13 B16 B20 B24 B28 B31:B32 B36 C36:C41 B43 C43:C48 B50 C50:C55 B57 C57:C62 B64 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C34" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(début v3): dernières modifications nécessaire avant de commencer à instancier
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11D3FA3D-D46F-41E6-8E5F-2DF762D19B16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E5412CE-1CEE-43F2-AA5D-3B92B9592498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34635" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3900" yWindow="1995" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$71</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$68</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="62">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -53,9 +53,6 @@
     <t>Experts </t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Chef.fe de Projet</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
   </si>
   <si>
     <t>Sources, liens, références, commits …</t>
-  </si>
-  <si>
-    <t>Introduction</t>
   </si>
   <si>
     <t>Bilan du jour :</t>
@@ -148,45 +142,18 @@
     <t>Visual Studio</t>
   </si>
   <si>
-    <t>Création et début de rédaction des méthodes pour le choix de tours et déplacement d'ennemi</t>
-  </si>
-  <si>
     <t>Création de tout les éléments nécessaires à la création du projet</t>
   </si>
   <si>
     <t>Commencement de la rédaction du code avec les fonctions de choix de placement des tours + déplacement des ennemis</t>
   </si>
   <si>
-    <t>Création du fichier Vscode et réflexion sur la manière d'aborder les premières fonctions</t>
-  </si>
-  <si>
-    <t>Finir d'implémenter la fonctionnalité de déplacement des tours</t>
-  </si>
-  <si>
-    <t xml:space="preserve">continuer le déplacement d'un ennemi avec plusieurs essais et complication  </t>
-  </si>
-  <si>
     <t xml:space="preserve">Avancée dans la rédaction des deux premières fonctions du code </t>
   </si>
   <si>
     <t>Avancée dans la rédaction des fonctions DeplacerEnnemis et TirerTour</t>
   </si>
   <si>
-    <t>Finir d'implémenter la fonctionnalité qui permet le déplacement d'un ennemi</t>
-  </si>
-  <si>
-    <t>début de rédaction de la méthode servant à tirer sur les ennemis avec les tours</t>
-  </si>
-  <si>
-    <t>Finir d'implémenter la fonctionnalité qui permet au tour de tirer sur les ennemis</t>
-  </si>
-  <si>
-    <t>En parallèle faire la dernière fonctionnalité servant à compter les dégats " CalculerDegats "</t>
-  </si>
-  <si>
-    <t>Finir d'implémenter la fonctionnalité qui permet de calculer les dégats infligés aux ennemis</t>
-  </si>
-  <si>
     <t>Avancée dans la rédaction des fonctions TirerTour et CalculerDegats</t>
   </si>
   <si>
@@ -205,21 +172,6 @@
     <t>Rendu de la v1</t>
   </si>
   <si>
-    <t>Mise en place de nouvelle classe et amélioration du code dans certaines fonctionnalités</t>
-  </si>
-  <si>
-    <t>Implémentation du projectile de la tour</t>
-  </si>
-  <si>
-    <t>Rendu v2</t>
-  </si>
-  <si>
-    <t>Rendu v1</t>
-  </si>
-  <si>
-    <t>Validation des dernières modifs pour la v1</t>
-  </si>
-  <si>
     <t>Realease v1 GitHub</t>
   </si>
   <si>
@@ -230,6 +182,276 @@
   </si>
   <si>
     <t>Amélioration de l'intro + Mise en page</t>
+  </si>
+  <si>
+    <t>Jonathan Melly</t>
+  </si>
+  <si>
+    <t>Création du fichier VScode et réflexion sur la manière d'aborder les premières fonctions</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Finir d'implémenter la fonctionnalité de déplacement des tours </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(terminé)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Création et début de rédaction des méthodes pour le choix de tours et déplacement d'ennemi </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(en cours)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Finir d'implémenter la fonctionnalité qui permet le déplacement d'un ennemi </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(terminé)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">début de rédaction de la méthode servant à tirer sur les ennemis avec les tours </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(en cours)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">continuer le déplacement d'un ennemi avec plusieurs essais et complication </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(en cours)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Finir d'implémenter la fonctionnalité qui permet au tour de tirer sur les ennemis </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(terminé)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">En parallèle faire la dernière fonctionnalité servant à compter les dégats " CalculerDegats " </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(en cours)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Finir d'implémenter la fonctionnalité qui permet de calculer les dégats infligés aux ennemis </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(terminé)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Validation des dernières modifs pour la v1 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(terminé)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Rendu v1 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(livrée)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Rendu v2 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(livrée)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Mise en place de nouvelles classes</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(HUD, Menu, et WinCondition)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>contenues dans un nouveau sous-namespace (Display)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>et amélioration du code dans certaines classes. (TowerManager).</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (terminée)</t>
+    </r>
+  </si>
+  <si>
+    <t>Excel</t>
+  </si>
+  <si>
+    <r>
+      <t>correction et amélioration du document avec les éléments demandés dans la critique du 17.02.2026</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (terminée)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">mise à jour de tout les fichiers .cs du projet en implémentant les cartouches demandées dans la critique du 17.02.2026 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(terminée) </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Implémentation du projectile de la tour grâce à une nouvelle classe et de nouvelles méthodes </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(en cours)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -301,7 +523,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -479,6 +701,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -488,7 +747,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -607,23 +866,67 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -941,7 +1244,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" style="1" customWidth="1"/>
@@ -958,814 +1261,837 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="35"/>
+      <c r="B1" s="38" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="38"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="18"/>
+      <c r="E1" s="18">
+        <f>C68</f>
+        <v>20.200000000000003</v>
+      </c>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="35" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="35"/>
+      <c r="B2" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="38"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="38"/>
+      <c r="D3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="35" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="35"/>
-      <c r="D3" s="20" t="s">
-        <v>6</v>
-      </c>
       <c r="E3" s="17" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="36" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37"/>
-      <c r="E4" s="38"/>
+        <v>6</v>
+      </c>
+      <c r="B4" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" s="30">
+        <v>25</v>
+      </c>
+      <c r="B6" s="42">
         <v>45671</v>
       </c>
       <c r="C6" s="5">
         <v>3</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E6" s="21"/>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B7" s="31"/>
+        <v>28</v>
+      </c>
+      <c r="B7" s="43"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E7" s="8"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="31"/>
+        <v>21</v>
+      </c>
+      <c r="B8" s="43"/>
       <c r="C8" s="8">
         <v>3</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E8" s="8"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="31"/>
+        <v>23</v>
+      </c>
+      <c r="B9" s="43"/>
       <c r="C9" s="8">
         <v>1</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="31"/>
+        <v>29</v>
+      </c>
+      <c r="B10" s="43"/>
       <c r="C10" s="10">
         <v>2</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B11" s="43"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
       </c>
-      <c r="D11" s="25"/>
-      <c r="E11" s="26"/>
+      <c r="D11" s="33"/>
+      <c r="E11" s="34"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="27" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="28"/>
-      <c r="E12" s="29"/>
-    </row>
-    <row r="13" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="B12" s="44"/>
+      <c r="C12" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="36"/>
+      <c r="E12" s="37"/>
+    </row>
+    <row r="13" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="30">
+        <v>29</v>
+      </c>
+      <c r="B13" s="42">
         <v>45678</v>
       </c>
       <c r="C13" s="5">
         <v>6</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B14" s="43"/>
       <c r="C14" s="22">
         <f>SUM(C13:C13)</f>
         <v>6</v>
       </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="26"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="34"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="27" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="28"/>
-      <c r="E15" s="29"/>
+        <v>11</v>
+      </c>
+      <c r="B15" s="44"/>
+      <c r="C15" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="36"/>
+      <c r="E15" s="37"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B16" s="30">
+        <v>29</v>
+      </c>
+      <c r="B16" s="42">
         <v>45681</v>
       </c>
       <c r="C16" s="5">
         <v>4</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="E16" s="21"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B17" s="31"/>
+        <v>29</v>
+      </c>
+      <c r="B17" s="43"/>
       <c r="C17" s="8">
         <v>2</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B18" s="43"/>
       <c r="C18" s="22">
         <f>SUM(C16:C17)</f>
         <v>6</v>
       </c>
-      <c r="D18" s="25"/>
-      <c r="E18" s="26"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="34"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="D19" s="28"/>
-      <c r="E19" s="29"/>
+        <v>11</v>
+      </c>
+      <c r="B19" s="44"/>
+      <c r="C19" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="36"/>
+      <c r="E19" s="37"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" s="30">
+        <v>29</v>
+      </c>
+      <c r="B20" s="42">
         <v>45682</v>
       </c>
       <c r="C20" s="5">
         <v>4</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="E20" s="21"/>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="31"/>
+        <v>29</v>
+      </c>
+      <c r="B21" s="43"/>
       <c r="C21" s="8">
         <v>2</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B22" s="43"/>
       <c r="C22" s="22">
         <f>SUM(C20:C21)</f>
         <v>6</v>
       </c>
-      <c r="D22" s="25"/>
-      <c r="E22" s="26"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="34"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B23" s="32"/>
-      <c r="C23" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="D23" s="28"/>
-      <c r="E23" s="29"/>
+        <v>11</v>
+      </c>
+      <c r="B23" s="44"/>
+      <c r="C23" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="D23" s="36"/>
+      <c r="E23" s="37"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" s="30">
+        <v>29</v>
+      </c>
+      <c r="B24" s="42">
         <v>46048</v>
       </c>
       <c r="C24" s="5">
         <v>2</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E24" s="21"/>
     </row>
-    <row r="25" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="31"/>
+        <v>29</v>
+      </c>
+      <c r="B25" s="43"/>
       <c r="C25" s="8">
         <v>2</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B26" s="43"/>
       <c r="C26" s="22">
         <f>SUM(C24:C25)</f>
         <v>4</v>
       </c>
-      <c r="D26" s="25"/>
-      <c r="E26" s="26"/>
+      <c r="D26" s="33"/>
+      <c r="E26" s="34"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="27" t="s">
-        <v>45</v>
-      </c>
-      <c r="D27" s="28"/>
-      <c r="E27" s="29"/>
-    </row>
-    <row r="28" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="B27" s="44"/>
+      <c r="C27" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="D27" s="36"/>
+      <c r="E27" s="37"/>
+    </row>
+    <row r="28" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B28" s="30">
+        <v>29</v>
+      </c>
+      <c r="B28" s="42">
         <v>46049</v>
       </c>
       <c r="C28" s="5">
         <v>2</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="E28" s="21"/>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B29" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B29" s="43"/>
       <c r="C29" s="22">
         <f>SUM(C28:C28)</f>
         <v>2</v>
       </c>
-      <c r="D29" s="25"/>
-      <c r="E29" s="26"/>
+      <c r="D29" s="33"/>
+      <c r="E29" s="34"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="27" t="s">
-        <v>46</v>
-      </c>
-      <c r="D30" s="28"/>
-      <c r="E30" s="29"/>
+        <v>11</v>
+      </c>
+      <c r="B30" s="44"/>
+      <c r="C30" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="D30" s="36"/>
+      <c r="E30" s="37"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B31" s="30">
+        <v>29</v>
+      </c>
+      <c r="B31" s="42">
         <v>46050</v>
       </c>
       <c r="C31" s="5">
         <v>6</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B32" s="31"/>
+        <v>28</v>
+      </c>
+      <c r="B32" s="43"/>
       <c r="C32" s="23">
         <v>1</v>
       </c>
       <c r="D32" s="24" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B33" s="31"/>
+        <v>29</v>
+      </c>
+      <c r="B33" s="43"/>
       <c r="C33" s="8">
         <v>5</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B34" s="31"/>
+        <v>20</v>
+      </c>
+      <c r="B34" s="43"/>
       <c r="C34" s="22">
         <f>SUM(C31:C33)</f>
         <v>12</v>
       </c>
-      <c r="D34" s="25"/>
-      <c r="E34" s="26"/>
+      <c r="D34" s="33"/>
+      <c r="E34" s="34"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B35" s="32"/>
-      <c r="C35" s="27" t="s">
-        <v>50</v>
-      </c>
-      <c r="D35" s="28"/>
-      <c r="E35" s="29"/>
-    </row>
-    <row r="36" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="B35" s="44"/>
+      <c r="C35" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="D35" s="36"/>
+      <c r="E35" s="37"/>
+    </row>
+    <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B36" s="30">
+        <v>29</v>
+      </c>
+      <c r="B36" s="47">
         <v>46057</v>
       </c>
       <c r="C36" s="5">
         <v>6</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="7"/>
-      <c r="B37" s="31"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="9"/>
-      <c r="E37" s="8"/>
-    </row>
-    <row r="38" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="7"/>
-      <c r="B38" s="31"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="8"/>
-    </row>
-    <row r="39" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="7"/>
-      <c r="B39" s="31"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="8"/>
-    </row>
-    <row r="40" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="10"/>
-      <c r="B40" s="31"/>
-      <c r="C40" s="10"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="10"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B37" s="48"/>
+      <c r="C37" s="22">
+        <f>SUM(C36:C36)</f>
+        <v>6</v>
+      </c>
+      <c r="D37" s="33"/>
+      <c r="E37" s="34"/>
+    </row>
+    <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" s="49"/>
+      <c r="C38" s="35"/>
+      <c r="D38" s="36"/>
+      <c r="E38" s="37"/>
+    </row>
+    <row r="39" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B39" s="42">
+        <v>46062</v>
+      </c>
+      <c r="C39" s="5">
+        <v>9</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B40" s="43"/>
+      <c r="C40" s="8">
+        <v>1</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B41" s="31"/>
-      <c r="C41" s="22">
-        <f>SUM(C36:C40)</f>
+      <c r="A41" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B41" s="43"/>
+      <c r="C41" s="8">
+        <v>2</v>
+      </c>
+      <c r="D41" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E41" s="8"/>
+    </row>
+    <row r="42" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B42" s="43"/>
+      <c r="C42" s="22">
+        <f>SUM(C39:C41)</f>
+        <v>12</v>
+      </c>
+      <c r="D42" s="33"/>
+      <c r="E42" s="34"/>
+    </row>
+    <row r="43" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B43" s="44"/>
+      <c r="C43" s="35"/>
+      <c r="D43" s="36"/>
+      <c r="E43" s="37"/>
+    </row>
+    <row r="44" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B44" s="42">
+        <v>46064</v>
+      </c>
+      <c r="C44" s="5">
+        <v>9</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E44" s="21"/>
+    </row>
+    <row r="45" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" s="43"/>
+      <c r="C45" s="22">
+        <f>SUM(C44:C44)</f>
+        <v>9</v>
+      </c>
+      <c r="D45" s="33"/>
+      <c r="E45" s="34"/>
+    </row>
+    <row r="46" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" s="44"/>
+      <c r="C46" s="35"/>
+      <c r="D46" s="36"/>
+      <c r="E46" s="37"/>
+    </row>
+    <row r="47" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A47" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B47" s="42">
+        <v>46076</v>
+      </c>
+      <c r="C47" s="5">
+        <v>4</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E47" s="21"/>
+    </row>
+    <row r="48" spans="1:5" ht="27" x14ac:dyDescent="0.25">
+      <c r="A48" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B48" s="43"/>
+      <c r="C48" s="8">
+        <v>2</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E48" s="8"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="7"/>
+      <c r="B49" s="43"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="8"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="7"/>
+      <c r="B50" s="43"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="8"/>
+    </row>
+    <row r="51" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="10"/>
+      <c r="B51" s="43"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="11"/>
+      <c r="E51" s="10"/>
+    </row>
+    <row r="52" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" s="43"/>
+      <c r="C52" s="22">
+        <f>SUM(C47:C51)</f>
         <v>6</v>
       </c>
-      <c r="D41" s="25"/>
-      <c r="E41" s="26"/>
-    </row>
-    <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="12" t="s">
+      <c r="D52" s="33"/>
+      <c r="E52" s="34"/>
+    </row>
+    <row r="53" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B53" s="44"/>
+      <c r="C53" s="35"/>
+      <c r="D53" s="36"/>
+      <c r="E53" s="37"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="4"/>
+      <c r="B54" s="30"/>
+      <c r="C54" s="5"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="21"/>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="7"/>
+      <c r="B55" s="31"/>
+      <c r="C55" s="8"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="8"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="7"/>
+      <c r="B56" s="31"/>
+      <c r="C56" s="8"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="8"/>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="7"/>
+      <c r="B57" s="31"/>
+      <c r="C57" s="8"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="8"/>
+    </row>
+    <row r="58" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="10"/>
+      <c r="B58" s="31"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="10"/>
+    </row>
+    <row r="59" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B59" s="31"/>
+      <c r="C59" s="22">
+        <f>SUM(C54:C58)</f>
+        <v>0</v>
+      </c>
+      <c r="D59" s="25"/>
+      <c r="E59" s="26"/>
+    </row>
+    <row r="60" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B60" s="32"/>
+      <c r="C60" s="27"/>
+      <c r="D60" s="28"/>
+      <c r="E60" s="29"/>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="4"/>
+      <c r="B61" s="30"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="6"/>
+      <c r="E61" s="21"/>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="7"/>
+      <c r="B62" s="31"/>
+      <c r="C62" s="8"/>
+      <c r="D62" s="9"/>
+      <c r="E62" s="8"/>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="7"/>
+      <c r="B63" s="31"/>
+      <c r="C63" s="8"/>
+      <c r="D63" s="9"/>
+      <c r="E63" s="8"/>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="7"/>
+      <c r="B64" s="31"/>
+      <c r="C64" s="8"/>
+      <c r="D64" s="9"/>
+      <c r="E64" s="8"/>
+    </row>
+    <row r="65" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="10"/>
+      <c r="B65" s="31"/>
+      <c r="C65" s="10"/>
+      <c r="D65" s="11"/>
+      <c r="E65" s="10"/>
+    </row>
+    <row r="66" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B66" s="31"/>
+      <c r="C66" s="22">
+        <f>SUM(C61:C65)</f>
+        <v>0</v>
+      </c>
+      <c r="D66" s="25"/>
+      <c r="E66" s="26"/>
+    </row>
+    <row r="67" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B67" s="32"/>
+      <c r="C67" s="27"/>
+      <c r="D67" s="28"/>
+      <c r="E67" s="29"/>
+    </row>
+    <row r="68" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="B68" s="46"/>
+      <c r="C68" s="13">
+        <f>MROUND(SUM(C6:C60) /8,0.2)</f>
+        <v>20.200000000000003</v>
+      </c>
+      <c r="D68" s="14"/>
+      <c r="E68" s="15"/>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B42" s="32"/>
-      <c r="C42" s="27"/>
-      <c r="D42" s="28"/>
-      <c r="E42" s="29"/>
-    </row>
-    <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B43" s="30">
-        <v>46062</v>
-      </c>
-      <c r="C43" s="5">
-        <v>9</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B44" s="31"/>
-      <c r="C44" s="8">
-        <v>1</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="E44" s="10" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="B45" s="31"/>
-      <c r="C45" s="8">
-        <v>2</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="E45" s="8"/>
-    </row>
-    <row r="46" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="7"/>
-      <c r="B46" s="31"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="8"/>
-    </row>
-    <row r="47" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="10"/>
-      <c r="B47" s="31"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="10"/>
-    </row>
-    <row r="48" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B48" s="31"/>
-      <c r="C48" s="22">
-        <f>SUM(C43:C47)</f>
-        <v>12</v>
-      </c>
-      <c r="D48" s="25"/>
-      <c r="E48" s="26"/>
-    </row>
-    <row r="49" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B49" s="32"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="28"/>
-      <c r="E49" s="29"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B50" s="30">
-        <v>46064</v>
-      </c>
-      <c r="C50" s="5">
-        <v>9</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="E50" s="21"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="7"/>
-      <c r="B51" s="31"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="9"/>
-      <c r="E51" s="8"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="7"/>
-      <c r="B52" s="31"/>
-      <c r="C52" s="8"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="8"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="7"/>
-      <c r="B53" s="31"/>
-      <c r="C53" s="8"/>
-      <c r="D53" s="9"/>
-      <c r="E53" s="8"/>
-    </row>
-    <row r="54" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="10"/>
-      <c r="B54" s="31"/>
-      <c r="C54" s="10"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="10"/>
-    </row>
-    <row r="55" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B55" s="31"/>
-      <c r="C55" s="22">
-        <f>SUM(C50:C54)</f>
-        <v>9</v>
-      </c>
-      <c r="D55" s="25"/>
-      <c r="E55" s="26"/>
-    </row>
-    <row r="56" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B56" s="32"/>
-      <c r="C56" s="27"/>
-      <c r="D56" s="28"/>
-      <c r="E56" s="29"/>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B57" s="30"/>
-      <c r="C57" s="5"/>
-      <c r="D57" s="6"/>
-      <c r="E57" s="21"/>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="7"/>
-      <c r="B58" s="31"/>
-      <c r="C58" s="8"/>
-      <c r="D58" s="9"/>
-      <c r="E58" s="8"/>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="7"/>
-      <c r="B59" s="31"/>
-      <c r="C59" s="8"/>
-      <c r="D59" s="9"/>
-      <c r="E59" s="8"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="7"/>
-      <c r="B60" s="31"/>
-      <c r="C60" s="8"/>
-      <c r="D60" s="9"/>
-      <c r="E60" s="8"/>
-    </row>
-    <row r="61" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="10"/>
-      <c r="B61" s="31"/>
-      <c r="C61" s="10"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="10"/>
-    </row>
-    <row r="62" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B62" s="31"/>
-      <c r="C62" s="22">
-        <f>SUM(C57:C61)</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="25"/>
-      <c r="E62" s="26"/>
-    </row>
-    <row r="63" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B63" s="32"/>
-      <c r="C63" s="27"/>
-      <c r="D63" s="28"/>
-      <c r="E63" s="29"/>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="4"/>
-      <c r="B64" s="30"/>
-      <c r="C64" s="5"/>
-      <c r="D64" s="6"/>
-      <c r="E64" s="21"/>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="7"/>
-      <c r="B65" s="31"/>
-      <c r="C65" s="8"/>
-      <c r="D65" s="9"/>
-      <c r="E65" s="8"/>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="7"/>
-      <c r="B66" s="31"/>
-      <c r="C66" s="8"/>
-      <c r="D66" s="9"/>
-      <c r="E66" s="8"/>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="7"/>
-      <c r="B67" s="31"/>
-      <c r="C67" s="8"/>
-      <c r="D67" s="9"/>
-      <c r="E67" s="8"/>
-    </row>
-    <row r="68" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="10"/>
-      <c r="B68" s="31"/>
-      <c r="C68" s="10"/>
-      <c r="D68" s="11"/>
-      <c r="E68" s="10"/>
-    </row>
-    <row r="69" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B69" s="31"/>
-      <c r="C69" s="22">
-        <f>SUM(C64:C68)</f>
-        <v>0</v>
-      </c>
-      <c r="D69" s="25"/>
-      <c r="E69" s="26"/>
-    </row>
-    <row r="70" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B70" s="32"/>
-      <c r="C70" s="27"/>
-      <c r="D70" s="28"/>
-      <c r="E70" s="29"/>
-    </row>
-    <row r="71" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="33" t="s">
-        <v>14</v>
-      </c>
-      <c r="B71" s="34"/>
-      <c r="C71" s="13">
-        <f>MROUND(SUM(C6:C70) /8,0.2)</f>
-        <v>18.8</v>
-      </c>
-      <c r="D71" s="14"/>
-      <c r="E71" s="15"/>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="16" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="16"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="41">
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="C42:E42"/>
+  <mergeCells count="38">
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="C46:E46"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="B39:B43"/>
+    <mergeCell ref="B47:B53"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="C38:E38"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -1780,34 +2106,9 @@
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="C19:E19"/>
-    <mergeCell ref="A71:B71"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B35"/>
-    <mergeCell ref="B36:B42"/>
-    <mergeCell ref="B43:B49"/>
-    <mergeCell ref="B57:B63"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="C49:E49"/>
-    <mergeCell ref="B50:B56"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="C56:E56"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="C63:E63"/>
-    <mergeCell ref="B64:B70"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="C70:E70"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C64:C69 B13 B16 B20 B24 B28 B31:B32 B36 C36:C41 B43 C43:C48 B50 C50:C55 B57 C57:C62 B64 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C34" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C39:C42 B13 B16 B20 B24 B28 B31:B32 B36 B39 B44 B47 C47:C52 C44:C45 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C34 C36:C37 C54:C59 B54 C61:C66 B61" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -1823,6 +2124,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -1984,12 +2291,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2000,6 +2301,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2017,15 +2327,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat(début des instances et de l'encapsulation): création des instances et début de l'encapsulation avec beaucoup de difficulté
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E5412CE-1CEE-43F2-AA5D-3B92B9592498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368E64B5-6687-4917-BBE9-060077CAE3B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="1995" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="64">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t>Explications / Etats</t>
-  </si>
-  <si>
-    <t>Sources, liens, références, commits …</t>
   </si>
   <si>
     <t>Bilan du jour :</t>
@@ -453,12 +450,32 @@
       <t>(en cours)</t>
     </r>
   </si>
+  <si>
+    <t>Difficulté, références, commits …</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difficulté à changer tout cela + Commit réalisé </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">commencement de la transformation du code en instance et encapsulation </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(en cours)</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Century Gothic"/>
@@ -502,6 +519,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -747,7 +771,7 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -866,23 +890,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -898,33 +920,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -1262,7 +1258,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="38" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C1" s="38"/>
       <c r="D1" s="20" t="s">
@@ -1270,7 +1266,7 @@
       </c>
       <c r="E1" s="18">
         <f>C68</f>
-        <v>20.200000000000003</v>
+        <v>23.200000000000003</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -1278,14 +1274,14 @@
         <v>2</v>
       </c>
       <c r="B2" s="38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" s="38"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1293,14 +1289,14 @@
         <v>4</v>
       </c>
       <c r="B3" s="38" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" s="38"/>
       <c r="D3" s="20" t="s">
         <v>5</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -1308,7 +1304,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C4" s="40"/>
       <c r="D4" s="40"/>
@@ -1322,714 +1318,726 @@
         <v>8</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>10</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="42">
+        <v>24</v>
+      </c>
+      <c r="B6" s="30">
         <v>45671</v>
       </c>
       <c r="C6" s="5">
         <v>3</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E6" s="21"/>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="43"/>
+        <v>27</v>
+      </c>
+      <c r="B7" s="31"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" s="8"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="43"/>
+        <v>20</v>
+      </c>
+      <c r="B8" s="31"/>
       <c r="C8" s="8">
         <v>3</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="8"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="43"/>
+        <v>22</v>
+      </c>
+      <c r="B9" s="31"/>
       <c r="C9" s="8">
         <v>1</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="43"/>
+        <v>28</v>
+      </c>
+      <c r="B10" s="31"/>
       <c r="C10" s="10">
         <v>2</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B11" s="31"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
       </c>
-      <c r="D11" s="33"/>
-      <c r="E11" s="34"/>
+      <c r="D11" s="25"/>
+      <c r="E11" s="26"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" s="44"/>
-      <c r="C12" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="36"/>
-      <c r="E12" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B12" s="32"/>
+      <c r="C12" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="28"/>
+      <c r="E12" s="29"/>
     </row>
     <row r="13" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="42">
+        <v>28</v>
+      </c>
+      <c r="B13" s="30">
         <v>45678</v>
       </c>
       <c r="C13" s="5">
         <v>6</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B14" s="31"/>
       <c r="C14" s="22">
         <f>SUM(C13:C13)</f>
         <v>6</v>
       </c>
-      <c r="D14" s="33"/>
-      <c r="E14" s="34"/>
+      <c r="D14" s="25"/>
+      <c r="E14" s="26"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="44"/>
-      <c r="C15" s="35" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B15" s="32"/>
+      <c r="C15" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="D15" s="28"/>
+      <c r="E15" s="29"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="42">
+        <v>28</v>
+      </c>
+      <c r="B16" s="30">
         <v>45681</v>
       </c>
       <c r="C16" s="5">
         <v>4</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E16" s="21"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17" s="43"/>
+        <v>28</v>
+      </c>
+      <c r="B17" s="31"/>
       <c r="C17" s="8">
         <v>2</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B18" s="31"/>
       <c r="C18" s="22">
         <f>SUM(C16:C17)</f>
         <v>6</v>
       </c>
-      <c r="D18" s="33"/>
-      <c r="E18" s="34"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="26"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B19" s="44"/>
-      <c r="C19" s="35" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B19" s="32"/>
+      <c r="C19" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="28"/>
+      <c r="E19" s="29"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="42">
+        <v>28</v>
+      </c>
+      <c r="B20" s="30">
         <v>45682</v>
       </c>
       <c r="C20" s="5">
         <v>4</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E20" s="21"/>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B21" s="43"/>
+        <v>28</v>
+      </c>
+      <c r="B21" s="31"/>
       <c r="C21" s="8">
         <v>2</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B22" s="31"/>
       <c r="C22" s="22">
         <f>SUM(C20:C21)</f>
         <v>6</v>
       </c>
-      <c r="D22" s="33"/>
-      <c r="E22" s="34"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="26"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B23" s="44"/>
-      <c r="C23" s="35" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B23" s="32"/>
+      <c r="C23" s="27" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="28"/>
+      <c r="E23" s="29"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B24" s="42">
+        <v>28</v>
+      </c>
+      <c r="B24" s="30">
         <v>46048</v>
       </c>
       <c r="C24" s="5">
         <v>2</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E24" s="21"/>
     </row>
     <row r="25" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="43"/>
+        <v>28</v>
+      </c>
+      <c r="B25" s="31"/>
       <c r="C25" s="8">
         <v>2</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B26" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B26" s="31"/>
       <c r="C26" s="22">
         <f>SUM(C24:C25)</f>
         <v>4</v>
       </c>
-      <c r="D26" s="33"/>
-      <c r="E26" s="34"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="26"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" s="44"/>
-      <c r="C27" s="35" t="s">
-        <v>34</v>
-      </c>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B27" s="32"/>
+      <c r="C27" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="28"/>
+      <c r="E27" s="29"/>
     </row>
     <row r="28" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="42">
+        <v>28</v>
+      </c>
+      <c r="B28" s="30">
         <v>46049</v>
       </c>
       <c r="C28" s="5">
         <v>2</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E28" s="21"/>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B29" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B29" s="31"/>
       <c r="C29" s="22">
         <f>SUM(C28:C28)</f>
         <v>2</v>
       </c>
-      <c r="D29" s="33"/>
-      <c r="E29" s="34"/>
+      <c r="D29" s="25"/>
+      <c r="E29" s="26"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B30" s="44"/>
-      <c r="C30" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="D30" s="36"/>
-      <c r="E30" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B30" s="32"/>
+      <c r="C30" s="27" t="s">
+        <v>34</v>
+      </c>
+      <c r="D30" s="28"/>
+      <c r="E30" s="29"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B31" s="42">
+        <v>28</v>
+      </c>
+      <c r="B31" s="30">
         <v>46050</v>
       </c>
       <c r="C31" s="5">
         <v>6</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B32" s="43"/>
+        <v>27</v>
+      </c>
+      <c r="B32" s="31"/>
       <c r="C32" s="23">
         <v>1</v>
       </c>
       <c r="D32" s="24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B33" s="43"/>
+        <v>28</v>
+      </c>
+      <c r="B33" s="31"/>
       <c r="C33" s="8">
         <v>5</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B34" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B34" s="31"/>
       <c r="C34" s="22">
         <f>SUM(C31:C33)</f>
         <v>12</v>
       </c>
-      <c r="D34" s="33"/>
-      <c r="E34" s="34"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="26"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B35" s="44"/>
-      <c r="C35" s="35" t="s">
-        <v>39</v>
-      </c>
-      <c r="D35" s="36"/>
-      <c r="E35" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B35" s="32"/>
+      <c r="C35" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="D35" s="28"/>
+      <c r="E35" s="29"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B36" s="47">
+        <v>28</v>
+      </c>
+      <c r="B36" s="35">
         <v>46057</v>
       </c>
       <c r="C36" s="5">
         <v>6</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B37" s="48"/>
+        <v>19</v>
+      </c>
+      <c r="B37" s="36"/>
       <c r="C37" s="22">
         <f>SUM(C36:C36)</f>
         <v>6</v>
       </c>
-      <c r="D37" s="33"/>
-      <c r="E37" s="34"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="26"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B38" s="49"/>
-      <c r="C38" s="35"/>
-      <c r="D38" s="36"/>
-      <c r="E38" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B38" s="37"/>
+      <c r="C38" s="27"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="29"/>
     </row>
     <row r="39" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B39" s="42">
+        <v>28</v>
+      </c>
+      <c r="B39" s="30">
         <v>46062</v>
       </c>
       <c r="C39" s="5">
         <v>9</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B40" s="43"/>
+        <v>27</v>
+      </c>
+      <c r="B40" s="31"/>
       <c r="C40" s="8">
         <v>1</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="B41" s="43"/>
+        <v>41</v>
+      </c>
+      <c r="B41" s="31"/>
       <c r="C41" s="8">
         <v>2</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E41" s="8"/>
     </row>
     <row r="42" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B42" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B42" s="31"/>
       <c r="C42" s="22">
         <f>SUM(C39:C41)</f>
         <v>12</v>
       </c>
-      <c r="D42" s="33"/>
-      <c r="E42" s="34"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="26"/>
     </row>
     <row r="43" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B43" s="44"/>
-      <c r="C43" s="35"/>
-      <c r="D43" s="36"/>
-      <c r="E43" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B43" s="32"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="29"/>
     </row>
     <row r="44" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B44" s="42">
+        <v>28</v>
+      </c>
+      <c r="B44" s="30">
         <v>46064</v>
       </c>
       <c r="C44" s="5">
         <v>9</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E44" s="21"/>
+        <v>60</v>
+      </c>
+      <c r="E44" s="42" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="45" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B45" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B45" s="31"/>
       <c r="C45" s="22">
         <f>SUM(C44:C44)</f>
         <v>9</v>
       </c>
-      <c r="D45" s="33"/>
-      <c r="E45" s="34"/>
+      <c r="D45" s="25"/>
+      <c r="E45" s="26"/>
     </row>
     <row r="46" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B46" s="44"/>
-      <c r="C46" s="35"/>
-      <c r="D46" s="36"/>
-      <c r="E46" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B46" s="32"/>
+      <c r="C46" s="27"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="29"/>
     </row>
     <row r="47" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B47" s="42">
+        <v>57</v>
+      </c>
+      <c r="B47" s="30">
         <v>46076</v>
       </c>
       <c r="C47" s="5">
         <v>4</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E47" s="21"/>
     </row>
     <row r="48" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B48" s="43"/>
+        <v>28</v>
+      </c>
+      <c r="B48" s="31"/>
       <c r="C48" s="8">
         <v>2</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E48" s="8"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="43"/>
+      <c r="B49" s="31"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="43"/>
+      <c r="B50" s="31"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
-      <c r="B51" s="43"/>
+      <c r="B51" s="31"/>
       <c r="C51" s="10"/>
       <c r="D51" s="11"/>
       <c r="E51" s="10"/>
     </row>
     <row r="52" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B52" s="43"/>
+        <v>19</v>
+      </c>
+      <c r="B52" s="31"/>
       <c r="C52" s="22">
         <f>SUM(C47:C51)</f>
         <v>6</v>
       </c>
-      <c r="D52" s="33"/>
-      <c r="E52" s="34"/>
+      <c r="D52" s="25"/>
+      <c r="E52" s="26"/>
     </row>
     <row r="53" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B53" s="44"/>
-      <c r="C53" s="35"/>
-      <c r="D53" s="36"/>
-      <c r="E53" s="37"/>
+        <v>10</v>
+      </c>
+      <c r="B53" s="32"/>
+      <c r="C53" s="27"/>
+      <c r="D53" s="28"/>
+      <c r="E53" s="29"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="4"/>
-      <c r="B54" s="30"/>
-      <c r="C54" s="5"/>
-      <c r="D54" s="6"/>
-      <c r="E54" s="21"/>
+      <c r="A54" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B54" s="35">
+        <v>46078</v>
+      </c>
+      <c r="C54" s="5">
+        <v>12</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E54" s="8" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="31"/>
+      <c r="B55" s="36"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="31"/>
+      <c r="B56" s="36"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="31"/>
+      <c r="B57" s="36"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="10"/>
-      <c r="B58" s="31"/>
+      <c r="B58" s="36"/>
       <c r="C58" s="10"/>
       <c r="D58" s="11"/>
       <c r="E58" s="10"/>
     </row>
     <row r="59" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B59" s="31"/>
+        <v>19</v>
+      </c>
+      <c r="B59" s="36"/>
       <c r="C59" s="22">
         <f>SUM(C54:C58)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D59" s="25"/>
       <c r="E59" s="26"/>
     </row>
     <row r="60" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B60" s="32"/>
+        <v>10</v>
+      </c>
+      <c r="B60" s="37"/>
       <c r="C60" s="27"/>
       <c r="D60" s="28"/>
       <c r="E60" s="29"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="4"/>
-      <c r="B61" s="30"/>
+      <c r="B61" s="35"/>
       <c r="C61" s="5"/>
       <c r="D61" s="6"/>
       <c r="E61" s="21"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="31"/>
+      <c r="B62" s="36"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="31"/>
+      <c r="B63" s="36"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="31"/>
+      <c r="B64" s="36"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="10"/>
-      <c r="B65" s="31"/>
+      <c r="B65" s="36"/>
       <c r="C65" s="10"/>
       <c r="D65" s="11"/>
       <c r="E65" s="10"/>
     </row>
     <row r="66" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B66" s="31"/>
+        <v>19</v>
+      </c>
+      <c r="B66" s="36"/>
       <c r="C66" s="22">
         <f>SUM(C61:C65)</f>
         <v>0</v>
@@ -2039,57 +2047,39 @@
     </row>
     <row r="67" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B67" s="32"/>
+        <v>10</v>
+      </c>
+      <c r="B67" s="37"/>
       <c r="C67" s="27"/>
       <c r="D67" s="28"/>
       <c r="E67" s="29"/>
     </row>
     <row r="68" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="B68" s="46"/>
+      <c r="A68" s="33" t="s">
+        <v>11</v>
+      </c>
+      <c r="B68" s="34"/>
       <c r="C68" s="13">
         <f>MROUND(SUM(C6:C60) /8,0.2)</f>
-        <v>20.200000000000003</v>
+        <v>23.200000000000003</v>
       </c>
       <c r="D68" s="14"/>
       <c r="E68" s="15"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="38">
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="C46:E46"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B35"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="B39:B43"/>
-    <mergeCell ref="B47:B53"/>
+  <mergeCells count="44">
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="C67:E67"/>
     <mergeCell ref="D37:E37"/>
     <mergeCell ref="C38:E38"/>
     <mergeCell ref="B1:C1"/>
@@ -2106,9 +2096,33 @@
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="C19:E19"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="B39:B43"/>
+    <mergeCell ref="B47:B53"/>
+    <mergeCell ref="B54:B60"/>
+    <mergeCell ref="B61:B67"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="C46:E46"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C39:C42 B13 B16 B20 B24 B28 B31:B32 B36 B39 B44 B47 C47:C52 C44:C45 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C34 C36:C37 C54:C59 B54 C61:C66 B61" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C39:C42 B13 B16 B20 B24 B28 B31:B32 B36 B39 B44 B47 C47:C52 C44:C45 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C34 C36:C37 C54:C59 B61 C61:C66" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -2124,12 +2138,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2291,6 +2299,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2301,15 +2315,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2327,6 +2332,15 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat(instanciation & encapsulation): mise en place de toutes les instances et encapsulation
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{368E64B5-6687-4917-BBE9-060077CAE3B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5626855E-CEDD-4F9D-8F5E-6A1B13A34F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3915" yWindow="2550" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="67">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -468,6 +468,37 @@
         <family val="2"/>
       </rPr>
       <t>(en cours)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Fin de la transformation de la totalité du code en instance avec de l'encapsulation</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (terminée)</t>
+    </r>
+  </si>
+  <si>
+    <t>Beaucoup de difficulté rencontrée mais objectif atteint</t>
+  </si>
+  <si>
+    <r>
+      <t>début de la rédaction de la comparaison entre les trois différentes versions du projet</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (en cours)</t>
     </r>
   </si>
 </sst>
@@ -858,6 +889,22 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -866,17 +913,11 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -890,12 +931,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -919,10 +954,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1247,7 +1278,7 @@
     <col min="2" max="2" width="14.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="20.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="91.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="53" style="1" customWidth="1"/>
     <col min="6" max="6" width="19.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="36" style="1" customWidth="1"/>
     <col min="8" max="16384" width="11.42578125" style="1"/>
@@ -1257,10 +1288,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="39" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="38"/>
+      <c r="C1" s="39"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -1273,10 +1304,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="38"/>
+      <c r="C2" s="39"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -1288,10 +1319,10 @@
       <c r="A3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="38" t="s">
+      <c r="B3" s="39" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="38"/>
+      <c r="C3" s="39"/>
       <c r="D3" s="20" t="s">
         <v>5</v>
       </c>
@@ -1303,12 +1334,12 @@
       <c r="A4" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="39" t="s">
+      <c r="B4" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1331,7 +1362,7 @@
       <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="30">
+      <c r="B6" s="33">
         <v>45671</v>
       </c>
       <c r="C6" s="5">
@@ -1346,7 +1377,7 @@
       <c r="A7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="31"/>
+      <c r="B7" s="34"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -1359,7 +1390,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="31"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="8">
         <v>3</v>
       </c>
@@ -1372,7 +1403,7 @@
       <c r="A9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="31"/>
+      <c r="B9" s="34"/>
       <c r="C9" s="8">
         <v>1</v>
       </c>
@@ -1385,7 +1416,7 @@
       <c r="A10" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="31"/>
+      <c r="B10" s="34"/>
       <c r="C10" s="10">
         <v>2</v>
       </c>
@@ -1400,30 +1431,30 @@
       <c r="A11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="31"/>
+      <c r="B11" s="34"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
       </c>
-      <c r="D11" s="25"/>
-      <c r="E11" s="26"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="30"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="27" t="s">
+      <c r="B12" s="35"/>
+      <c r="C12" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="28"/>
-      <c r="E12" s="29"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="28"/>
     </row>
     <row r="13" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="30">
+      <c r="B13" s="33">
         <v>45678</v>
       </c>
       <c r="C13" s="5">
@@ -1440,30 +1471,30 @@
       <c r="A14" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="31"/>
+      <c r="B14" s="34"/>
       <c r="C14" s="22">
         <f>SUM(C13:C13)</f>
         <v>6</v>
       </c>
-      <c r="D14" s="25"/>
-      <c r="E14" s="26"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="32"/>
-      <c r="C15" s="27" t="s">
+      <c r="B15" s="35"/>
+      <c r="C15" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="D15" s="28"/>
-      <c r="E15" s="29"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="28"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="30">
+      <c r="B16" s="33">
         <v>45681</v>
       </c>
       <c r="C16" s="5">
@@ -1478,7 +1509,7 @@
       <c r="A17" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="31"/>
+      <c r="B17" s="34"/>
       <c r="C17" s="8">
         <v>2</v>
       </c>
@@ -1491,30 +1522,30 @@
       <c r="A18" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="31"/>
+      <c r="B18" s="34"/>
       <c r="C18" s="22">
         <f>SUM(C16:C17)</f>
         <v>6</v>
       </c>
-      <c r="D18" s="25"/>
-      <c r="E18" s="26"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="30"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="27" t="s">
+      <c r="B19" s="35"/>
+      <c r="C19" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="28"/>
-      <c r="E19" s="29"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="28"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="30">
+      <c r="B20" s="33">
         <v>45682</v>
       </c>
       <c r="C20" s="5">
@@ -1529,7 +1560,7 @@
       <c r="A21" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="31"/>
+      <c r="B21" s="34"/>
       <c r="C21" s="8">
         <v>2</v>
       </c>
@@ -1542,30 +1573,30 @@
       <c r="A22" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="31"/>
+      <c r="B22" s="34"/>
       <c r="C22" s="22">
         <f>SUM(C20:C21)</f>
         <v>6</v>
       </c>
-      <c r="D22" s="25"/>
-      <c r="E22" s="26"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="30"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="32"/>
-      <c r="C23" s="27" t="s">
+      <c r="B23" s="35"/>
+      <c r="C23" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="28"/>
-      <c r="E23" s="29"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="28"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="30">
+      <c r="B24" s="33">
         <v>46048</v>
       </c>
       <c r="C24" s="5">
@@ -1580,7 +1611,7 @@
       <c r="A25" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="31"/>
+      <c r="B25" s="34"/>
       <c r="C25" s="8">
         <v>2</v>
       </c>
@@ -1593,30 +1624,30 @@
       <c r="A26" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="31"/>
+      <c r="B26" s="34"/>
       <c r="C26" s="22">
         <f>SUM(C24:C25)</f>
         <v>4</v>
       </c>
-      <c r="D26" s="25"/>
-      <c r="E26" s="26"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="30"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="32"/>
-      <c r="C27" s="27" t="s">
+      <c r="B27" s="35"/>
+      <c r="C27" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="D27" s="28"/>
-      <c r="E27" s="29"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="28"/>
     </row>
     <row r="28" spans="1:5" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="30">
+      <c r="B28" s="33">
         <v>46049</v>
       </c>
       <c r="C28" s="5">
@@ -1631,30 +1662,30 @@
       <c r="A29" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="31"/>
+      <c r="B29" s="34"/>
       <c r="C29" s="22">
         <f>SUM(C28:C28)</f>
         <v>2</v>
       </c>
-      <c r="D29" s="25"/>
-      <c r="E29" s="26"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="30"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="27" t="s">
+      <c r="B30" s="35"/>
+      <c r="C30" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="D30" s="28"/>
-      <c r="E30" s="29"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="28"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="30">
+      <c r="B31" s="33">
         <v>46050</v>
       </c>
       <c r="C31" s="5">
@@ -1671,7 +1702,7 @@
       <c r="A32" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B32" s="31"/>
+      <c r="B32" s="34"/>
       <c r="C32" s="23">
         <v>1</v>
       </c>
@@ -1686,7 +1717,7 @@
       <c r="A33" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="31"/>
+      <c r="B33" s="34"/>
       <c r="C33" s="8">
         <v>5</v>
       </c>
@@ -1701,30 +1732,30 @@
       <c r="A34" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B34" s="31"/>
+      <c r="B34" s="34"/>
       <c r="C34" s="22">
         <f>SUM(C31:C33)</f>
         <v>12</v>
       </c>
-      <c r="D34" s="25"/>
-      <c r="E34" s="26"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="30"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B35" s="32"/>
-      <c r="C35" s="27" t="s">
+      <c r="B35" s="35"/>
+      <c r="C35" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="D35" s="28"/>
-      <c r="E35" s="29"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="28"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B36" s="35">
+      <c r="B36" s="36">
         <v>46057</v>
       </c>
       <c r="C36" s="5">
@@ -1741,28 +1772,28 @@
       <c r="A37" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B37" s="36"/>
+      <c r="B37" s="37"/>
       <c r="C37" s="22">
         <f>SUM(C36:C36)</f>
         <v>6</v>
       </c>
-      <c r="D37" s="25"/>
-      <c r="E37" s="26"/>
+      <c r="D37" s="29"/>
+      <c r="E37" s="30"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="37"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="28"/>
-      <c r="E38" s="29"/>
+      <c r="B38" s="38"/>
+      <c r="C38" s="26"/>
+      <c r="D38" s="27"/>
+      <c r="E38" s="28"/>
     </row>
     <row r="39" spans="1:5" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B39" s="30">
+      <c r="B39" s="33">
         <v>46062</v>
       </c>
       <c r="C39" s="5">
@@ -1779,7 +1810,7 @@
       <c r="A40" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B40" s="31"/>
+      <c r="B40" s="34"/>
       <c r="C40" s="8">
         <v>1</v>
       </c>
@@ -1794,7 +1825,7 @@
       <c r="A41" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B41" s="31"/>
+      <c r="B41" s="34"/>
       <c r="C41" s="8">
         <v>2</v>
       </c>
@@ -1807,28 +1838,28 @@
       <c r="A42" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B42" s="31"/>
+      <c r="B42" s="34"/>
       <c r="C42" s="22">
         <f>SUM(C39:C41)</f>
         <v>12</v>
       </c>
-      <c r="D42" s="25"/>
-      <c r="E42" s="26"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="30"/>
     </row>
     <row r="43" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B43" s="32"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="28"/>
-      <c r="E43" s="29"/>
+      <c r="B43" s="35"/>
+      <c r="C43" s="26"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="28"/>
     </row>
     <row r="44" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="30">
+      <c r="B44" s="33">
         <v>46064</v>
       </c>
       <c r="C44" s="5">
@@ -1837,7 +1868,7 @@
       <c r="D44" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E44" s="42" t="s">
+      <c r="E44" s="25" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1845,28 +1876,28 @@
       <c r="A45" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B45" s="31"/>
+      <c r="B45" s="34"/>
       <c r="C45" s="22">
         <f>SUM(C44:C44)</f>
         <v>9</v>
       </c>
-      <c r="D45" s="25"/>
-      <c r="E45" s="26"/>
+      <c r="D45" s="29"/>
+      <c r="E45" s="30"/>
     </row>
     <row r="46" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B46" s="32"/>
-      <c r="C46" s="27"/>
-      <c r="D46" s="28"/>
-      <c r="E46" s="29"/>
+      <c r="B46" s="35"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="28"/>
     </row>
     <row r="47" spans="1:5" ht="27" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B47" s="30">
+      <c r="B47" s="33">
         <v>46076</v>
       </c>
       <c r="C47" s="5">
@@ -1881,7 +1912,7 @@
       <c r="A48" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="31"/>
+      <c r="B48" s="34"/>
       <c r="C48" s="8">
         <v>2</v>
       </c>
@@ -1892,21 +1923,21 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="31"/>
+      <c r="B49" s="34"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="31"/>
+      <c r="B50" s="34"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
-      <c r="B51" s="31"/>
+      <c r="B51" s="34"/>
       <c r="C51" s="10"/>
       <c r="D51" s="11"/>
       <c r="E51" s="10"/>
@@ -1915,28 +1946,28 @@
       <c r="A52" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B52" s="31"/>
+      <c r="B52" s="34"/>
       <c r="C52" s="22">
         <f>SUM(C47:C51)</f>
         <v>6</v>
       </c>
-      <c r="D52" s="25"/>
-      <c r="E52" s="26"/>
+      <c r="D52" s="29"/>
+      <c r="E52" s="30"/>
     </row>
     <row r="53" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B53" s="32"/>
-      <c r="C53" s="27"/>
-      <c r="D53" s="28"/>
-      <c r="E53" s="29"/>
+      <c r="B53" s="35"/>
+      <c r="C53" s="26"/>
+      <c r="D53" s="27"/>
+      <c r="E53" s="28"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B54" s="35">
+      <c r="B54" s="36">
         <v>46078</v>
       </c>
       <c r="C54" s="5">
@@ -1951,28 +1982,28 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="36"/>
+      <c r="B55" s="37"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="36"/>
+      <c r="B56" s="37"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="36"/>
+      <c r="B57" s="37"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="10"/>
-      <c r="B58" s="36"/>
+      <c r="B58" s="37"/>
       <c r="C58" s="10"/>
       <c r="D58" s="11"/>
       <c r="E58" s="10"/>
@@ -1981,54 +2012,70 @@
       <c r="A59" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B59" s="36"/>
+      <c r="B59" s="37"/>
       <c r="C59" s="22">
         <f>SUM(C54:C58)</f>
         <v>12</v>
       </c>
-      <c r="D59" s="25"/>
-      <c r="E59" s="26"/>
+      <c r="D59" s="29"/>
+      <c r="E59" s="30"/>
     </row>
     <row r="60" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B60" s="37"/>
-      <c r="C60" s="27"/>
-      <c r="D60" s="28"/>
-      <c r="E60" s="29"/>
+      <c r="B60" s="38"/>
+      <c r="C60" s="26"/>
+      <c r="D60" s="27"/>
+      <c r="E60" s="28"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="4"/>
-      <c r="B61" s="35"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="6"/>
-      <c r="E61" s="21"/>
+      <c r="A61" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B61" s="36">
+        <v>46085</v>
+      </c>
+      <c r="C61" s="5">
+        <v>10</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E61" s="25" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="7"/>
-      <c r="B62" s="36"/>
-      <c r="C62" s="8"/>
-      <c r="D62" s="9"/>
+      <c r="A62" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B62" s="37"/>
+      <c r="C62" s="8">
+        <v>1</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="36"/>
+      <c r="B63" s="37"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="36"/>
+      <c r="B64" s="37"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="10"/>
-      <c r="B65" s="36"/>
+      <c r="B65" s="37"/>
       <c r="C65" s="10"/>
       <c r="D65" s="11"/>
       <c r="E65" s="10"/>
@@ -2037,28 +2084,28 @@
       <c r="A66" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B66" s="36"/>
+      <c r="B66" s="37"/>
       <c r="C66" s="22">
         <f>SUM(C61:C65)</f>
-        <v>0</v>
-      </c>
-      <c r="D66" s="25"/>
-      <c r="E66" s="26"/>
+        <v>11</v>
+      </c>
+      <c r="D66" s="29"/>
+      <c r="E66" s="30"/>
     </row>
     <row r="67" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B67" s="37"/>
-      <c r="C67" s="27"/>
-      <c r="D67" s="28"/>
-      <c r="E67" s="29"/>
+      <c r="B67" s="38"/>
+      <c r="C67" s="26"/>
+      <c r="D67" s="27"/>
+      <c r="E67" s="28"/>
     </row>
     <row r="68" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="33" t="s">
+      <c r="A68" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="B68" s="34"/>
+      <c r="B68" s="32"/>
       <c r="C68" s="13">
         <f>MROUND(SUM(C6:C60) /8,0.2)</f>
         <v>23.200000000000003</v>
@@ -2082,6 +2129,12 @@
     <mergeCell ref="C67:E67"/>
     <mergeCell ref="D37:E37"/>
     <mergeCell ref="C38:E38"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="C46:E46"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -2096,6 +2149,8 @@
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="C19:E19"/>
+    <mergeCell ref="B20:B23"/>
+    <mergeCell ref="D22:E22"/>
     <mergeCell ref="A68:B68"/>
     <mergeCell ref="B24:B27"/>
     <mergeCell ref="B28:B30"/>
@@ -2105,21 +2160,13 @@
     <mergeCell ref="B47:B53"/>
     <mergeCell ref="B54:B60"/>
     <mergeCell ref="B61:B67"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="B44:B46"/>
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="D26:E26"/>
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="C30:E30"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="C46:E46"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C39:C42 B13 B16 B20 B24 B28 B31:B32 B36 B39 B44 B47 C47:C52 C44:C45 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C34 C36:C37 C54:C59 B61 C61:C66" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">

</xml_diff>

<commit_message>
feat(renommage): renommage de Enemy en Monster
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5626855E-CEDD-4F9D-8F5E-6A1B13A34F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFC6BA6-805D-48C2-8DB8-139AD33B08A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3915" yWindow="2550" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$68</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Journal!$A$1:$E$82</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="70">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -500,6 +500,15 @@
       </rPr>
       <t xml:space="preserve"> (en cours)</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Renommage de Enemy en Monster </t>
+  </si>
+  <si>
+    <t>Début de création de l'objet pour avoir plusieurs monstre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">beaucoup de difficulté car ne comprend pas très bien </t>
   </si>
 </sst>
 </file>
@@ -913,11 +922,17 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -931,6 +946,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -942,18 +963,6 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1271,7 +1280,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" style="1" customWidth="1"/>
@@ -1288,15 +1297,15 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="39"/>
+      <c r="C1" s="31"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="18">
-        <f>C68</f>
+        <f>C82</f>
         <v>23.200000000000003</v>
       </c>
     </row>
@@ -1304,10 +1313,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="39"/>
+      <c r="C2" s="31"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -1319,10 +1328,10 @@
       <c r="A3" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="39" t="s">
+      <c r="B3" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="39"/>
+      <c r="C3" s="31"/>
       <c r="D3" s="20" t="s">
         <v>5</v>
       </c>
@@ -1334,12 +1343,12 @@
       <c r="A4" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="40" t="s">
+      <c r="B4" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="41"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="42"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="34"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -1362,7 +1371,7 @@
       <c r="A6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="35">
         <v>45671</v>
       </c>
       <c r="C6" s="5">
@@ -1377,7 +1386,7 @@
       <c r="A7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="34"/>
+      <c r="B7" s="36"/>
       <c r="C7" s="8">
         <v>3</v>
       </c>
@@ -1390,7 +1399,7 @@
       <c r="A8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="34"/>
+      <c r="B8" s="36"/>
       <c r="C8" s="8">
         <v>3</v>
       </c>
@@ -1403,7 +1412,7 @@
       <c r="A9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="34"/>
+      <c r="B9" s="36"/>
       <c r="C9" s="8">
         <v>1</v>
       </c>
@@ -1416,7 +1425,7 @@
       <c r="A10" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="34"/>
+      <c r="B10" s="36"/>
       <c r="C10" s="10">
         <v>2</v>
       </c>
@@ -1431,7 +1440,7 @@
       <c r="A11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="34"/>
+      <c r="B11" s="36"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>12</v>
@@ -1443,7 +1452,7 @@
       <c r="A12" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="35"/>
+      <c r="B12" s="37"/>
       <c r="C12" s="26" t="s">
         <v>29</v>
       </c>
@@ -1454,7 +1463,7 @@
       <c r="A13" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="33">
+      <c r="B13" s="35">
         <v>45678</v>
       </c>
       <c r="C13" s="5">
@@ -1471,7 +1480,7 @@
       <c r="A14" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="34"/>
+      <c r="B14" s="36"/>
       <c r="C14" s="22">
         <f>SUM(C13:C13)</f>
         <v>6</v>
@@ -1483,7 +1492,7 @@
       <c r="A15" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B15" s="35"/>
+      <c r="B15" s="37"/>
       <c r="C15" s="26" t="s">
         <v>30</v>
       </c>
@@ -1494,7 +1503,7 @@
       <c r="A16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="33">
+      <c r="B16" s="35">
         <v>45681</v>
       </c>
       <c r="C16" s="5">
@@ -1509,7 +1518,7 @@
       <c r="A17" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="34"/>
+      <c r="B17" s="36"/>
       <c r="C17" s="8">
         <v>2</v>
       </c>
@@ -1522,7 +1531,7 @@
       <c r="A18" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="34"/>
+      <c r="B18" s="36"/>
       <c r="C18" s="22">
         <f>SUM(C16:C17)</f>
         <v>6</v>
@@ -1534,7 +1543,7 @@
       <c r="A19" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="35"/>
+      <c r="B19" s="37"/>
       <c r="C19" s="26" t="s">
         <v>31</v>
       </c>
@@ -1545,7 +1554,7 @@
       <c r="A20" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="35">
         <v>45682</v>
       </c>
       <c r="C20" s="5">
@@ -1560,7 +1569,7 @@
       <c r="A21" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B21" s="34"/>
+      <c r="B21" s="36"/>
       <c r="C21" s="8">
         <v>2</v>
       </c>
@@ -1573,7 +1582,7 @@
       <c r="A22" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="34"/>
+      <c r="B22" s="36"/>
       <c r="C22" s="22">
         <f>SUM(C20:C21)</f>
         <v>6</v>
@@ -1585,7 +1594,7 @@
       <c r="A23" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="35"/>
+      <c r="B23" s="37"/>
       <c r="C23" s="26" t="s">
         <v>32</v>
       </c>
@@ -1596,7 +1605,7 @@
       <c r="A24" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="33">
+      <c r="B24" s="35">
         <v>46048</v>
       </c>
       <c r="C24" s="5">
@@ -1611,7 +1620,7 @@
       <c r="A25" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B25" s="34"/>
+      <c r="B25" s="36"/>
       <c r="C25" s="8">
         <v>2</v>
       </c>
@@ -1624,7 +1633,7 @@
       <c r="A26" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="34"/>
+      <c r="B26" s="36"/>
       <c r="C26" s="22">
         <f>SUM(C24:C25)</f>
         <v>4</v>
@@ -1636,7 +1645,7 @@
       <c r="A27" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B27" s="35"/>
+      <c r="B27" s="37"/>
       <c r="C27" s="26" t="s">
         <v>33</v>
       </c>
@@ -1647,7 +1656,7 @@
       <c r="A28" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B28" s="33">
+      <c r="B28" s="35">
         <v>46049</v>
       </c>
       <c r="C28" s="5">
@@ -1662,7 +1671,7 @@
       <c r="A29" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="34"/>
+      <c r="B29" s="36"/>
       <c r="C29" s="22">
         <f>SUM(C28:C28)</f>
         <v>2</v>
@@ -1674,7 +1683,7 @@
       <c r="A30" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B30" s="35"/>
+      <c r="B30" s="37"/>
       <c r="C30" s="26" t="s">
         <v>34</v>
       </c>
@@ -1685,7 +1694,7 @@
       <c r="A31" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="33">
+      <c r="B31" s="35">
         <v>46050</v>
       </c>
       <c r="C31" s="5">
@@ -1702,7 +1711,7 @@
       <c r="A32" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B32" s="34"/>
+      <c r="B32" s="36"/>
       <c r="C32" s="23">
         <v>1</v>
       </c>
@@ -1717,7 +1726,7 @@
       <c r="A33" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="34"/>
+      <c r="B33" s="36"/>
       <c r="C33" s="8">
         <v>5</v>
       </c>
@@ -1732,7 +1741,7 @@
       <c r="A34" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B34" s="34"/>
+      <c r="B34" s="36"/>
       <c r="C34" s="22">
         <f>SUM(C31:C33)</f>
         <v>12</v>
@@ -1744,7 +1753,7 @@
       <c r="A35" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B35" s="35"/>
+      <c r="B35" s="37"/>
       <c r="C35" s="26" t="s">
         <v>38</v>
       </c>
@@ -1755,7 +1764,7 @@
       <c r="A36" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B36" s="36">
+      <c r="B36" s="40">
         <v>46057</v>
       </c>
       <c r="C36" s="5">
@@ -1772,7 +1781,7 @@
       <c r="A37" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B37" s="37"/>
+      <c r="B37" s="41"/>
       <c r="C37" s="22">
         <f>SUM(C36:C36)</f>
         <v>6</v>
@@ -1784,7 +1793,7 @@
       <c r="A38" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B38" s="38"/>
+      <c r="B38" s="42"/>
       <c r="C38" s="26"/>
       <c r="D38" s="27"/>
       <c r="E38" s="28"/>
@@ -1793,7 +1802,7 @@
       <c r="A39" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B39" s="33">
+      <c r="B39" s="35">
         <v>46062</v>
       </c>
       <c r="C39" s="5">
@@ -1810,7 +1819,7 @@
       <c r="A40" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B40" s="34"/>
+      <c r="B40" s="36"/>
       <c r="C40" s="8">
         <v>1</v>
       </c>
@@ -1825,7 +1834,7 @@
       <c r="A41" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B41" s="34"/>
+      <c r="B41" s="36"/>
       <c r="C41" s="8">
         <v>2</v>
       </c>
@@ -1838,7 +1847,7 @@
       <c r="A42" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B42" s="34"/>
+      <c r="B42" s="36"/>
       <c r="C42" s="22">
         <f>SUM(C39:C41)</f>
         <v>12</v>
@@ -1850,7 +1859,7 @@
       <c r="A43" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B43" s="35"/>
+      <c r="B43" s="37"/>
       <c r="C43" s="26"/>
       <c r="D43" s="27"/>
       <c r="E43" s="28"/>
@@ -1859,7 +1868,7 @@
       <c r="A44" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="33">
+      <c r="B44" s="35">
         <v>46064</v>
       </c>
       <c r="C44" s="5">
@@ -1876,7 +1885,7 @@
       <c r="A45" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B45" s="34"/>
+      <c r="B45" s="36"/>
       <c r="C45" s="22">
         <f>SUM(C44:C44)</f>
         <v>9</v>
@@ -1888,7 +1897,7 @@
       <c r="A46" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B46" s="35"/>
+      <c r="B46" s="37"/>
       <c r="C46" s="26"/>
       <c r="D46" s="27"/>
       <c r="E46" s="28"/>
@@ -1897,7 +1906,7 @@
       <c r="A47" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B47" s="33">
+      <c r="B47" s="35">
         <v>46076</v>
       </c>
       <c r="C47" s="5">
@@ -1912,7 +1921,7 @@
       <c r="A48" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B48" s="34"/>
+      <c r="B48" s="36"/>
       <c r="C48" s="8">
         <v>2</v>
       </c>
@@ -1923,21 +1932,21 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
-      <c r="B49" s="34"/>
+      <c r="B49" s="36"/>
       <c r="C49" s="8"/>
       <c r="D49" s="9"/>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="34"/>
+      <c r="B50" s="36"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="10"/>
-      <c r="B51" s="34"/>
+      <c r="B51" s="36"/>
       <c r="C51" s="10"/>
       <c r="D51" s="11"/>
       <c r="E51" s="10"/>
@@ -1946,7 +1955,7 @@
       <c r="A52" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B52" s="34"/>
+      <c r="B52" s="36"/>
       <c r="C52" s="22">
         <f>SUM(C47:C51)</f>
         <v>6</v>
@@ -1958,7 +1967,7 @@
       <c r="A53" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B53" s="35"/>
+      <c r="B53" s="37"/>
       <c r="C53" s="26"/>
       <c r="D53" s="27"/>
       <c r="E53" s="28"/>
@@ -1967,7 +1976,7 @@
       <c r="A54" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B54" s="36">
+      <c r="B54" s="40">
         <v>46078</v>
       </c>
       <c r="C54" s="5">
@@ -1982,28 +1991,28 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="7"/>
-      <c r="B55" s="37"/>
+      <c r="B55" s="41"/>
       <c r="C55" s="8"/>
       <c r="D55" s="9"/>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="37"/>
+      <c r="B56" s="41"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="37"/>
+      <c r="B57" s="41"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="10"/>
-      <c r="B58" s="37"/>
+      <c r="B58" s="41"/>
       <c r="C58" s="10"/>
       <c r="D58" s="11"/>
       <c r="E58" s="10"/>
@@ -2012,7 +2021,7 @@
       <c r="A59" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B59" s="37"/>
+      <c r="B59" s="41"/>
       <c r="C59" s="22">
         <f>SUM(C54:C58)</f>
         <v>12</v>
@@ -2024,7 +2033,7 @@
       <c r="A60" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B60" s="38"/>
+      <c r="B60" s="42"/>
       <c r="C60" s="26"/>
       <c r="D60" s="27"/>
       <c r="E60" s="28"/>
@@ -2033,7 +2042,7 @@
       <c r="A61" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B61" s="36">
+      <c r="B61" s="40">
         <v>46085</v>
       </c>
       <c r="C61" s="5">
@@ -2050,7 +2059,7 @@
       <c r="A62" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B62" s="37"/>
+      <c r="B62" s="41"/>
       <c r="C62" s="8">
         <v>1</v>
       </c>
@@ -2061,21 +2070,21 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="37"/>
+      <c r="B63" s="41"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="37"/>
+      <c r="B64" s="41"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="10"/>
-      <c r="B65" s="37"/>
+      <c r="B65" s="41"/>
       <c r="C65" s="10"/>
       <c r="D65" s="11"/>
       <c r="E65" s="10"/>
@@ -2084,7 +2093,7 @@
       <c r="A66" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B66" s="37"/>
+      <c r="B66" s="41"/>
       <c r="C66" s="22">
         <f>SUM(C61:C65)</f>
         <v>11</v>
@@ -2096,45 +2105,193 @@
       <c r="A67" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B67" s="38"/>
+      <c r="B67" s="42"/>
       <c r="C67" s="26"/>
       <c r="D67" s="27"/>
       <c r="E67" s="28"/>
     </row>
-    <row r="68" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="31" t="s">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B68" s="40">
+        <v>46085</v>
+      </c>
+      <c r="C68" s="5">
+        <v>7</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E68" s="25"/>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B69" s="41"/>
+      <c r="C69" s="8">
+        <v>1</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="E69" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="7"/>
+      <c r="B70" s="41"/>
+      <c r="C70" s="8"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="8"/>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="7"/>
+      <c r="B71" s="41"/>
+      <c r="C71" s="8"/>
+      <c r="D71" s="9"/>
+      <c r="E71" s="8"/>
+    </row>
+    <row r="72" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="10"/>
+      <c r="B72" s="41"/>
+      <c r="C72" s="10"/>
+      <c r="D72" s="11"/>
+      <c r="E72" s="10"/>
+    </row>
+    <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B73" s="41"/>
+      <c r="C73" s="22">
+        <f>SUM(C68:C72)</f>
+        <v>8</v>
+      </c>
+      <c r="D73" s="29"/>
+      <c r="E73" s="30"/>
+    </row>
+    <row r="74" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B74" s="42"/>
+      <c r="C74" s="26"/>
+      <c r="D74" s="27"/>
+      <c r="E74" s="28"/>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B75" s="40">
+        <v>46085</v>
+      </c>
+      <c r="C75" s="5">
+        <v>10</v>
+      </c>
+      <c r="D75" s="6"/>
+      <c r="E75" s="25"/>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B76" s="41"/>
+      <c r="C76" s="8">
+        <v>1</v>
+      </c>
+      <c r="D76" s="9"/>
+      <c r="E76" s="8"/>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="7"/>
+      <c r="B77" s="41"/>
+      <c r="C77" s="8"/>
+      <c r="D77" s="9"/>
+      <c r="E77" s="8"/>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="7"/>
+      <c r="B78" s="41"/>
+      <c r="C78" s="8"/>
+      <c r="D78" s="9"/>
+      <c r="E78" s="8"/>
+    </row>
+    <row r="79" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="10"/>
+      <c r="B79" s="41"/>
+      <c r="C79" s="10"/>
+      <c r="D79" s="11"/>
+      <c r="E79" s="10"/>
+    </row>
+    <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B80" s="41"/>
+      <c r="C80" s="22">
+        <f>SUM(C75:C79)</f>
         <v>11</v>
       </c>
-      <c r="B68" s="32"/>
-      <c r="C68" s="13">
+      <c r="D80" s="29"/>
+      <c r="E80" s="30"/>
+    </row>
+    <row r="81" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B81" s="42"/>
+      <c r="C81" s="26"/>
+      <c r="D81" s="27"/>
+      <c r="E81" s="28"/>
+    </row>
+    <row r="82" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="B82" s="39"/>
+      <c r="C82" s="13">
         <f>MROUND(SUM(C6:C60) /8,0.2)</f>
         <v>23.200000000000003</v>
       </c>
-      <c r="D68" s="14"/>
-      <c r="E68" s="15"/>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="16" t="s">
+      <c r="D82" s="14"/>
+      <c r="E82" s="15"/>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="16"/>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="44">
-    <mergeCell ref="C60:E60"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="C67:E67"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="C53:E53"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="C43:E43"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="C46:E46"/>
+  <mergeCells count="50">
+    <mergeCell ref="D73:E73"/>
+    <mergeCell ref="C74:E74"/>
+    <mergeCell ref="B75:B81"/>
+    <mergeCell ref="D80:E80"/>
+    <mergeCell ref="C81:E81"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="A82:B82"/>
+    <mergeCell ref="B24:B27"/>
+    <mergeCell ref="B28:B30"/>
+    <mergeCell ref="B31:B35"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="B39:B43"/>
+    <mergeCell ref="B47:B53"/>
+    <mergeCell ref="B54:B60"/>
+    <mergeCell ref="B61:B67"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="B68:B74"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -2151,25 +2308,21 @@
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="B20:B23"/>
     <mergeCell ref="D22:E22"/>
-    <mergeCell ref="A68:B68"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B35"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="B39:B43"/>
-    <mergeCell ref="B47:B53"/>
-    <mergeCell ref="B54:B60"/>
-    <mergeCell ref="B61:B67"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="C27:E27"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="C67:E67"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="C43:E43"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="C46:E46"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C39:C42 B13 B16 B20 B24 B28 B31:B32 B36 B39 B44 B47 C47:C52 C44:C45 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C34 C36:C37 C54:C59 B61 C61:C66" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
+    <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6:C6 C39:C42 B13 B16 B20 B24 B28 B31:B32 B36 B39 B44 B47 C47:C52 C44:C45 C7:C11 C13:C14 C16:C18 C20:C22 C24:C26 C28:C29 C31:C34 C36:C37 C54:C59 B61 C61:C66 B68 C68:C73 B75 C75:C80" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -2185,6 +2338,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2346,12 +2505,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2362,6 +2515,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2379,15 +2541,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
feat(remis de la v3 finale): fin de la mise en place de la v3
</commit_message>
<xml_diff>
--- a/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
+++ b/doc/P-P_OO-LeoBouzon-jnltrav.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\I320\Projet\OO-them-ALL\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFC6BA6-805D-48C2-8DB8-139AD33B08A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93E535D1-5636-4485-A62D-BE3FE3C1A8FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6810" yWindow="1500" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="72">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -505,10 +505,49 @@
     <t xml:space="preserve">Renommage de Enemy en Monster </t>
   </si>
   <si>
-    <t>Début de création de l'objet pour avoir plusieurs monstre</t>
-  </si>
-  <si>
     <t xml:space="preserve">beaucoup de difficulté car ne comprend pas très bien </t>
+  </si>
+  <si>
+    <r>
+      <t>Début de création de l'objet pour avoir plusieurs monstre</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (en cours)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Fin de la création des deux monstres </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(terminée)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Implémentation du Boss pour avoir un héritage dans mon projet </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Century Gothic"/>
+        <family val="2"/>
+      </rPr>
+      <t>(terminée)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2115,10 +2154,10 @@
         <v>28</v>
       </c>
       <c r="B68" s="40">
-        <v>46085</v>
+        <v>46092</v>
       </c>
       <c r="C68" s="5">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D68" s="6" t="s">
         <v>67</v>
@@ -2127,17 +2166,17 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="B69" s="41"/>
       <c r="C69" s="8">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="D69" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E69" s="8" t="s">
         <v>68</v>
-      </c>
-      <c r="E69" s="8" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
@@ -2168,7 +2207,7 @@
       <c r="B73" s="41"/>
       <c r="C73" s="22">
         <f>SUM(C68:C72)</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D73" s="29"/>
       <c r="E73" s="30"/>
@@ -2183,27 +2222,31 @@
       <c r="E74" s="28"/>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="4" t="s">
+      <c r="A75" s="7" t="s">
         <v>28</v>
       </c>
       <c r="B75" s="40">
-        <v>46085</v>
+        <v>46094</v>
       </c>
       <c r="C75" s="5">
-        <v>10</v>
-      </c>
-      <c r="D75" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>70</v>
+      </c>
       <c r="E75" s="25"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="B76" s="41"/>
       <c r="C76" s="8">
-        <v>1</v>
-      </c>
-      <c r="D76" s="9"/>
+        <v>4</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>71</v>
+      </c>
       <c r="E76" s="8"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -2234,7 +2277,7 @@
       <c r="B80" s="41"/>
       <c r="C80" s="22">
         <f>SUM(C75:C79)</f>
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D80" s="29"/>
       <c r="E80" s="30"/>

</xml_diff>